<commit_message>
second part with examples
</commit_message>
<xml_diff>
--- a/StructureDefinition-ophthalmic-condition.xlsx
+++ b/StructureDefinition-ophthalmic-condition.xlsx
@@ -10,13 +10,13 @@
     <sheet name="Elements" r:id="rId4" sheetId="2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="true">Elements!$A$1:$AP$43</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="true">Elements!$A$1:$AP$47</definedName>
   </definedNames>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1662" uniqueCount="374">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1817" uniqueCount="393">
   <si>
     <t>Property</t>
   </si>
@@ -60,7 +60,7 @@
     <t>Date</t>
   </si>
   <si>
-    <t>2026-08-18T00:29:29+00:00</t>
+    <t>2026-08-18T20:04:06+00:00</t>
   </si>
   <si>
     <t>Publisher</t>
@@ -445,21 +445,21 @@
     <t>Condition.extension</t>
   </si>
   <si>
+    <t>extensions
+user content</t>
+  </si>
+  <si>
     <t xml:space="preserve">Extension
 </t>
   </si>
   <si>
-    <t>Extension</t>
-  </si>
-  <si>
-    <t>An Extension</t>
-  </si>
-  <si>
-    <t xml:space="preserve">value:url}
-</t>
-  </si>
-  <si>
-    <t>open</t>
+    <t>Additional content defined by implementations</t>
+  </si>
+  <si>
+    <t>May be used to represent additional information that is not part of the basic definition of the resource. To make the use of extensions safe and manageable, there is a strict set of governance  applied to the definition and use of extensions. Though any implementer can define an extension, there is a set of requirements that SHALL be met as part of the definition of the extension.</t>
+  </si>
+  <si>
+    <t>There can be no stigma associated with the use of extensions by any application, project, or standard - regardless of the institution or jurisdiction that uses or defines the extensions.  The use of extensions is what allows the FHIR specification to retain a core level of simplicity for everyone.</t>
   </si>
   <si>
     <t>DomainResource.extension</t>
@@ -469,105 +469,7 @@
 ext-1:Must have either extensions or value[x], not both {extension.exists() != value.exists()}</t>
   </si>
   <si>
-    <t>Condition.extension:bodySiteEye</t>
-  </si>
-  <si>
-    <t>bodySiteEye</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Extension {bodySite}
-</t>
-  </si>
-  <si>
-    <t>Laterality of the diagnosis, via BodyStructure</t>
-  </si>
-  <si>
-    <t>Record details about the anatomical location of a specimen or body part. This resource may be used when a coded concept does not provide the necessary detail needed for the use case.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">ele-1
-</t>
-  </si>
-  <si>
-    <t>Condition.extension:bodySiteEye.id</t>
-  </si>
-  <si>
-    <t>Condition.extension.id</t>
-  </si>
-  <si>
-    <t xml:space="preserve">string
-</t>
-  </si>
-  <si>
-    <t>Unique id for inter-element referencing</t>
-  </si>
-  <si>
-    <t>Unique id for the element within a resource (for internal references). This may be any string value that does not contain spaces.</t>
-  </si>
-  <si>
-    <t>Element.id</t>
-  </si>
-  <si>
-    <t>n/a</t>
-  </si>
-  <si>
-    <t>Condition.extension:bodySiteEye.extension</t>
-  </si>
-  <si>
-    <t>Condition.extension.extension</t>
-  </si>
-  <si>
-    <t>Extensions are always sliced by (at least) url</t>
-  </si>
-  <si>
-    <t>Element.extension</t>
-  </si>
-  <si>
-    <t>Condition.extension:bodySiteEye.url</t>
-  </si>
-  <si>
-    <t>Condition.extension.url</t>
-  </si>
-  <si>
-    <t>identifies the meaning of the extension</t>
-  </si>
-  <si>
-    <t>Source of the definition for the extension code - a logical name or a URL.</t>
-  </si>
-  <si>
-    <t>The definition may point directly to a computable or human-readable definition of the extensibility codes, or it may be a logical URI as declared in some other specification. The definition SHALL be a URI for the Structure Definition defining the extension.</t>
-  </si>
-  <si>
-    <t>http://hl7.org/fhir/StructureDefinition/bodySite</t>
-  </si>
-  <si>
-    <t>Extension.url</t>
-  </si>
-  <si>
-    <t>Condition.extension:bodySiteEye.value[x]</t>
-  </si>
-  <si>
-    <t>Condition.extension.value[x]</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Reference(https://YasniiSS.github.io/fhir4eyes/StructureDefinition/ocular-body-structure)
-</t>
-  </si>
-  <si>
-    <t>Value of extension</t>
-  </si>
-  <si>
-    <t>Value of extension - must be one of a constrained set of the data types (see [Extensibility](http://hl7.org/fhir/R4/extensibility.html) for a list).</t>
-  </si>
-  <si>
-    <t>Extension.value[x]</t>
-  </si>
-  <si>
     <t>Condition.modifierExtension</t>
-  </si>
-  <si>
-    <t>extensions
-user content</t>
   </si>
   <si>
     <t>Extensions that cannot be ignored</t>
@@ -577,9 +479,6 @@
 Modifier extensions SHALL NOT change the meaning of any elements on Resource or DomainResource (including cannot change the meaning of modifierExtension itself).</t>
   </si>
   <si>
-    <t>There can be no stigma associated with the use of extensions by any application, project, or standard - regardless of the institution or jurisdiction that uses or defines the extensions.  The use of extensions is what allows the FHIR specification to retain a core level of simplicity for everyone.</t>
-  </si>
-  <si>
     <t>Modifier extensions allow for extensions that *cannot* be safely ignored to be clearly distinguished from the vast majority of extensions which can be safely ignored.  This promotes interoperability by eliminating the need for implementers to prohibit the presence of extensions. For further information, see the [definition of modifier extensions](http://hl7.org/fhir/R4/extensibility.html#modifierExtension).</t>
   </si>
   <si>
@@ -593,7 +492,7 @@
 </t>
   </si>
   <si>
-    <t>External Ids for this condition</t>
+    <t>External identifier for this diagnosis, if applicable</t>
   </si>
   <si>
     <t>Business identifiers assigned to this condition by the performer or other systems which remain constant as the resource is updated and propagates from server to server.</t>
@@ -834,6 +733,170 @@
     <t>363698007</t>
   </si>
   <si>
+    <t>Condition.bodySite.id</t>
+  </si>
+  <si>
+    <t xml:space="preserve">string
+</t>
+  </si>
+  <si>
+    <t>Unique id for inter-element referencing</t>
+  </si>
+  <si>
+    <t>Unique id for the element within a resource (for internal references). This may be any string value that does not contain spaces.</t>
+  </si>
+  <si>
+    <t>Element.id</t>
+  </si>
+  <si>
+    <t>n/a</t>
+  </si>
+  <si>
+    <t>Condition.bodySite.extension</t>
+  </si>
+  <si>
+    <t>May be used to represent additional information that is not part of the basic definition of the element. To make the use of extensions safe and manageable, there is a strict set of governance  applied to the definition and use of extensions. Though any implementer can define an extension, there is a set of requirements that SHALL be met as part of the definition of the extension.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">value:url}
+</t>
+  </si>
+  <si>
+    <t>Extensions are always sliced by (at least) url</t>
+  </si>
+  <si>
+    <t>open</t>
+  </si>
+  <si>
+    <t>Element.extension</t>
+  </si>
+  <si>
+    <t>Condition.bodySite.extension:bodySiteEye</t>
+  </si>
+  <si>
+    <t>bodySiteEye</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Extension {bodySite}
+</t>
+  </si>
+  <si>
+    <t>Laterality of the diagnosis, via BodyStructure</t>
+  </si>
+  <si>
+    <t>Record details about the anatomical location of a specimen or body part. This resource may be used when a coded concept does not provide the necessary detail needed for the use case.</t>
+  </si>
+  <si>
+    <t>Condition.bodySite.extension:bodySiteEye.id</t>
+  </si>
+  <si>
+    <t>Condition.bodySite.extension.id</t>
+  </si>
+  <si>
+    <t>Condition.bodySite.extension:bodySiteEye.extension</t>
+  </si>
+  <si>
+    <t>Condition.bodySite.extension.extension</t>
+  </si>
+  <si>
+    <t>Extension</t>
+  </si>
+  <si>
+    <t>An Extension</t>
+  </si>
+  <si>
+    <t>Condition.bodySite.extension:bodySiteEye.url</t>
+  </si>
+  <si>
+    <t>Condition.bodySite.extension.url</t>
+  </si>
+  <si>
+    <t>identifies the meaning of the extension</t>
+  </si>
+  <si>
+    <t>Source of the definition for the extension code - a logical name or a URL.</t>
+  </si>
+  <si>
+    <t>The definition may point directly to a computable or human-readable definition of the extensibility codes, or it may be a logical URI as declared in some other specification. The definition SHALL be a URI for the Structure Definition defining the extension.</t>
+  </si>
+  <si>
+    <t>http://hl7.org/fhir/StructureDefinition/bodySite</t>
+  </si>
+  <si>
+    <t>Extension.url</t>
+  </si>
+  <si>
+    <t>Condition.bodySite.extension:bodySiteEye.value[x]</t>
+  </si>
+  <si>
+    <t>Condition.bodySite.extension.value[x]</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Reference(https://YasniiSS.github.io/fhir4eyes/StructureDefinition/ocular-body-structure)
+</t>
+  </si>
+  <si>
+    <t>Value of extension</t>
+  </si>
+  <si>
+    <t>Value of extension - must be one of a constrained set of the data types (see [Extensibility](http://hl7.org/fhir/R4/extensibility.html) for a list).</t>
+  </si>
+  <si>
+    <t>Extension.value[x]</t>
+  </si>
+  <si>
+    <t>Condition.bodySite.coding</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Coding
+</t>
+  </si>
+  <si>
+    <t>Code defined by a terminology system</t>
+  </si>
+  <si>
+    <t>A reference to a code defined by a terminology system.</t>
+  </si>
+  <si>
+    <t>Codes may be defined very casually in enumerations, or code lists, up to very formal definitions such as SNOMED CT - see the HL7 v3 Core Principles for more information.  Ordering of codings is undefined and SHALL NOT be used to infer meaning. Generally, at most only one of the coding values will be labeled as UserSelected = true.</t>
+  </si>
+  <si>
+    <t>Allows for alternative encodings within a code system, and translations to other code systems.</t>
+  </si>
+  <si>
+    <t>CodeableConcept.coding</t>
+  </si>
+  <si>
+    <t>C*E.1-8, C*E.10-22</t>
+  </si>
+  <si>
+    <t>union(., ./translation)</t>
+  </si>
+  <si>
+    <t>Condition.bodySite.text</t>
+  </si>
+  <si>
+    <t>Plain text representation of the concept</t>
+  </si>
+  <si>
+    <t>A human language representation of the concept as seen/selected/uttered by the user who entered the data and/or which represents the intended meaning of the user.</t>
+  </si>
+  <si>
+    <t>Very often the text is the same as a displayName of one of the codings.</t>
+  </si>
+  <si>
+    <t>The codes from the terminologies do not always capture the correct meaning with all the nuances of the human using them, or sometimes there is no appropriate code at all. In these cases, the text is used to capture the full meaning of the source.</t>
+  </si>
+  <si>
+    <t>CodeableConcept.text</t>
+  </si>
+  <si>
+    <t>C*E.9. But note many systems use C*E.2 for this</t>
+  </si>
+  <si>
+    <t>./originalText[mediaType/code="text/plain"]/data</t>
+  </si>
+  <si>
     <t>Condition.subject</t>
   </si>
   <si>
@@ -1027,12 +1090,6 @@
   </si>
   <si>
     <t>Condition.stage.extension</t>
-  </si>
-  <si>
-    <t>Additional content defined by implementations</t>
-  </si>
-  <si>
-    <t>May be used to represent additional information that is not part of the basic definition of the element. To make the use of extensions safe and manageable, there is a strict set of governance  applied to the definition and use of extensions. Though any implementer can define an extension, there is a set of requirements that SHALL be met as part of the definition of the extension.</t>
   </si>
   <si>
     <t>Condition.stage.modifierExtension</t>
@@ -1521,11 +1578,11 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <dimension ref="A1:AP43"/>
+  <dimension ref="A1:AP47"/>
   <sheetFormatPr defaultRowHeight="15.0"/>
   <cols>
-    <col min="1" max="1" width="35.09765625" customWidth="true" bestFit="true"/>
-    <col min="2" max="2" width="30.765625" customWidth="true" bestFit="true"/>
+    <col min="1" max="1" width="42.50390625" customWidth="true" bestFit="true"/>
+    <col min="2" max="2" width="32.1796875" customWidth="true" bestFit="true"/>
     <col min="3" max="3" width="10.8515625" customWidth="true" bestFit="true" hidden="true"/>
     <col min="4" max="4" width="34.21875" customWidth="true" bestFit="true" hidden="true"/>
     <col min="5" max="5" width="5.80859375" customWidth="true" bestFit="true"/>
@@ -2540,7 +2597,7 @@
       </c>
       <c r="C9" s="2"/>
       <c r="D9" t="s" s="2">
-        <v>80</v>
+        <v>137</v>
       </c>
       <c r="E9" s="2"/>
       <c r="F9" t="s" s="2">
@@ -2559,15 +2616,17 @@
         <v>80</v>
       </c>
       <c r="K9" t="s" s="2">
-        <v>137</v>
+        <v>138</v>
       </c>
       <c r="L9" t="s" s="2">
-        <v>138</v>
+        <v>139</v>
       </c>
       <c r="M9" t="s" s="2">
-        <v>139</v>
-      </c>
-      <c r="N9" s="2"/>
+        <v>140</v>
+      </c>
+      <c r="N9" t="s" s="2">
+        <v>141</v>
+      </c>
       <c r="O9" s="2"/>
       <c r="P9" t="s" s="2">
         <v>80</v>
@@ -2604,14 +2663,16 @@
         <v>80</v>
       </c>
       <c r="AB9" t="s" s="2">
-        <v>140</v>
-      </c>
-      <c r="AC9" s="2"/>
+        <v>80</v>
+      </c>
+      <c r="AC9" t="s" s="2">
+        <v>80</v>
+      </c>
       <c r="AD9" t="s" s="2">
         <v>80</v>
       </c>
       <c r="AE9" t="s" s="2">
-        <v>141</v>
+        <v>80</v>
       </c>
       <c r="AF9" t="s" s="2">
         <v>142</v>
@@ -2638,7 +2699,7 @@
         <v>80</v>
       </c>
       <c r="AN9" t="s" s="2">
-        <v>80</v>
+        <v>135</v>
       </c>
       <c r="AO9" t="s" s="2">
         <v>80</v>
@@ -2647,18 +2708,16 @@
         <v>80</v>
       </c>
     </row>
-    <row r="10">
+    <row r="10" hidden="true">
       <c r="A10" t="s" s="2">
         <v>144</v>
       </c>
       <c r="B10" t="s" s="2">
-        <v>136</v>
-      </c>
-      <c r="C10" t="s" s="2">
-        <v>145</v>
-      </c>
+        <v>144</v>
+      </c>
+      <c r="C10" s="2"/>
       <c r="D10" t="s" s="2">
-        <v>80</v>
+        <v>137</v>
       </c>
       <c r="E10" s="2"/>
       <c r="F10" t="s" s="2">
@@ -2668,25 +2727,29 @@
         <v>82</v>
       </c>
       <c r="H10" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="I10" t="s" s="2">
         <v>93</v>
       </c>
-      <c r="I10" t="s" s="2">
-        <v>80</v>
-      </c>
       <c r="J10" t="s" s="2">
         <v>80</v>
       </c>
       <c r="K10" t="s" s="2">
+        <v>138</v>
+      </c>
+      <c r="L10" t="s" s="2">
+        <v>145</v>
+      </c>
+      <c r="M10" t="s" s="2">
         <v>146</v>
       </c>
-      <c r="L10" t="s" s="2">
+      <c r="N10" t="s" s="2">
+        <v>141</v>
+      </c>
+      <c r="O10" t="s" s="2">
         <v>147</v>
       </c>
-      <c r="M10" t="s" s="2">
-        <v>148</v>
-      </c>
-      <c r="N10" s="2"/>
-      <c r="O10" s="2"/>
       <c r="P10" t="s" s="2">
         <v>80</v>
       </c>
@@ -2734,7 +2797,7 @@
         <v>80</v>
       </c>
       <c r="AF10" t="s" s="2">
-        <v>142</v>
+        <v>148</v>
       </c>
       <c r="AG10" t="s" s="2">
         <v>81</v>
@@ -2743,7 +2806,7 @@
         <v>82</v>
       </c>
       <c r="AI10" t="s" s="2">
-        <v>149</v>
+        <v>80</v>
       </c>
       <c r="AJ10" t="s" s="2">
         <v>143</v>
@@ -2758,7 +2821,7 @@
         <v>80</v>
       </c>
       <c r="AN10" t="s" s="2">
-        <v>80</v>
+        <v>135</v>
       </c>
       <c r="AO10" t="s" s="2">
         <v>80</v>
@@ -2767,12 +2830,12 @@
         <v>80</v>
       </c>
     </row>
-    <row r="11" hidden="true">
+    <row r="11">
       <c r="A11" t="s" s="2">
-        <v>150</v>
+        <v>149</v>
       </c>
       <c r="B11" t="s" s="2">
-        <v>151</v>
+        <v>149</v>
       </c>
       <c r="C11" s="2"/>
       <c r="D11" t="s" s="2">
@@ -2783,28 +2846,32 @@
         <v>81</v>
       </c>
       <c r="G11" t="s" s="2">
-        <v>92</v>
+        <v>82</v>
       </c>
       <c r="H11" t="s" s="2">
-        <v>80</v>
+        <v>93</v>
       </c>
       <c r="I11" t="s" s="2">
         <v>80</v>
       </c>
       <c r="J11" t="s" s="2">
-        <v>80</v>
+        <v>93</v>
       </c>
       <c r="K11" t="s" s="2">
+        <v>150</v>
+      </c>
+      <c r="L11" t="s" s="2">
+        <v>151</v>
+      </c>
+      <c r="M11" t="s" s="2">
         <v>152</v>
       </c>
-      <c r="L11" t="s" s="2">
+      <c r="N11" t="s" s="2">
         <v>153</v>
       </c>
-      <c r="M11" t="s" s="2">
+      <c r="O11" t="s" s="2">
         <v>154</v>
       </c>
-      <c r="N11" s="2"/>
-      <c r="O11" s="2"/>
       <c r="P11" t="s" s="2">
         <v>80</v>
       </c>
@@ -2852,22 +2919,22 @@
         <v>80</v>
       </c>
       <c r="AF11" t="s" s="2">
+        <v>149</v>
+      </c>
+      <c r="AG11" t="s" s="2">
+        <v>81</v>
+      </c>
+      <c r="AH11" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="AI11" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="AJ11" t="s" s="2">
+        <v>104</v>
+      </c>
+      <c r="AK11" t="s" s="2">
         <v>155</v>
-      </c>
-      <c r="AG11" t="s" s="2">
-        <v>81</v>
-      </c>
-      <c r="AH11" t="s" s="2">
-        <v>92</v>
-      </c>
-      <c r="AI11" t="s" s="2">
-        <v>80</v>
-      </c>
-      <c r="AJ11" t="s" s="2">
-        <v>80</v>
-      </c>
-      <c r="AK11" t="s" s="2">
-        <v>80</v>
       </c>
       <c r="AL11" t="s" s="2">
         <v>80</v>
@@ -2879,7 +2946,7 @@
         <v>156</v>
       </c>
       <c r="AO11" t="s" s="2">
-        <v>80</v>
+        <v>157</v>
       </c>
       <c r="AP11" t="s" s="2">
         <v>80</v>
@@ -2887,7 +2954,7 @@
     </row>
     <row r="12" hidden="true">
       <c r="A12" t="s" s="2">
-        <v>157</v>
+        <v>158</v>
       </c>
       <c r="B12" t="s" s="2">
         <v>158</v>
@@ -2901,27 +2968,29 @@
         <v>81</v>
       </c>
       <c r="G12" t="s" s="2">
-        <v>81</v>
+        <v>92</v>
       </c>
       <c r="H12" t="s" s="2">
         <v>80</v>
       </c>
       <c r="I12" t="s" s="2">
-        <v>80</v>
+        <v>93</v>
       </c>
       <c r="J12" t="s" s="2">
-        <v>80</v>
+        <v>93</v>
       </c>
       <c r="K12" t="s" s="2">
-        <v>137</v>
+        <v>159</v>
       </c>
       <c r="L12" t="s" s="2">
-        <v>138</v>
+        <v>160</v>
       </c>
       <c r="M12" t="s" s="2">
-        <v>139</v>
-      </c>
-      <c r="N12" s="2"/>
+        <v>161</v>
+      </c>
+      <c r="N12" t="s" s="2">
+        <v>162</v>
+      </c>
       <c r="O12" s="2"/>
       <c r="P12" t="s" s="2">
         <v>80</v>
@@ -2946,58 +3015,58 @@
         <v>80</v>
       </c>
       <c r="X12" t="s" s="2">
-        <v>80</v>
+        <v>163</v>
       </c>
       <c r="Y12" t="s" s="2">
-        <v>80</v>
+        <v>164</v>
       </c>
       <c r="Z12" t="s" s="2">
-        <v>80</v>
+        <v>165</v>
       </c>
       <c r="AA12" t="s" s="2">
         <v>80</v>
       </c>
       <c r="AB12" t="s" s="2">
-        <v>140</v>
+        <v>80</v>
       </c>
       <c r="AC12" t="s" s="2">
-        <v>159</v>
+        <v>80</v>
       </c>
       <c r="AD12" t="s" s="2">
         <v>80</v>
       </c>
       <c r="AE12" t="s" s="2">
-        <v>141</v>
+        <v>80</v>
       </c>
       <c r="AF12" t="s" s="2">
-        <v>160</v>
+        <v>158</v>
       </c>
       <c r="AG12" t="s" s="2">
         <v>81</v>
       </c>
       <c r="AH12" t="s" s="2">
-        <v>82</v>
+        <v>92</v>
       </c>
       <c r="AI12" t="s" s="2">
-        <v>80</v>
+        <v>166</v>
       </c>
       <c r="AJ12" t="s" s="2">
-        <v>143</v>
+        <v>104</v>
       </c>
       <c r="AK12" t="s" s="2">
-        <v>80</v>
+        <v>167</v>
       </c>
       <c r="AL12" t="s" s="2">
-        <v>80</v>
+        <v>168</v>
       </c>
       <c r="AM12" t="s" s="2">
-        <v>80</v>
+        <v>169</v>
       </c>
       <c r="AN12" t="s" s="2">
-        <v>80</v>
+        <v>170</v>
       </c>
       <c r="AO12" t="s" s="2">
-        <v>80</v>
+        <v>171</v>
       </c>
       <c r="AP12" t="s" s="2">
         <v>80</v>
@@ -3005,10 +3074,10 @@
     </row>
     <row r="13" hidden="true">
       <c r="A13" t="s" s="2">
-        <v>161</v>
+        <v>172</v>
       </c>
       <c r="B13" t="s" s="2">
-        <v>162</v>
+        <v>172</v>
       </c>
       <c r="C13" s="2"/>
       <c r="D13" t="s" s="2">
@@ -3016,7 +3085,7 @@
       </c>
       <c r="E13" s="2"/>
       <c r="F13" t="s" s="2">
-        <v>92</v>
+        <v>81</v>
       </c>
       <c r="G13" t="s" s="2">
         <v>92</v>
@@ -3025,22 +3094,22 @@
         <v>80</v>
       </c>
       <c r="I13" t="s" s="2">
-        <v>80</v>
+        <v>93</v>
       </c>
       <c r="J13" t="s" s="2">
-        <v>80</v>
+        <v>93</v>
       </c>
       <c r="K13" t="s" s="2">
-        <v>106</v>
+        <v>159</v>
       </c>
       <c r="L13" t="s" s="2">
-        <v>163</v>
+        <v>173</v>
       </c>
       <c r="M13" t="s" s="2">
-        <v>164</v>
+        <v>174</v>
       </c>
       <c r="N13" t="s" s="2">
-        <v>165</v>
+        <v>175</v>
       </c>
       <c r="O13" s="2"/>
       <c r="P13" t="s" s="2">
@@ -3048,7 +3117,7 @@
       </c>
       <c r="Q13" s="2"/>
       <c r="R13" t="s" s="2">
-        <v>166</v>
+        <v>80</v>
       </c>
       <c r="S13" t="s" s="2">
         <v>80</v>
@@ -3066,13 +3135,13 @@
         <v>80</v>
       </c>
       <c r="X13" t="s" s="2">
-        <v>80</v>
+        <v>163</v>
       </c>
       <c r="Y13" t="s" s="2">
-        <v>80</v>
+        <v>176</v>
       </c>
       <c r="Z13" t="s" s="2">
-        <v>80</v>
+        <v>177</v>
       </c>
       <c r="AA13" t="s" s="2">
         <v>80</v>
@@ -3090,45 +3159,45 @@
         <v>80</v>
       </c>
       <c r="AF13" t="s" s="2">
-        <v>167</v>
+        <v>172</v>
       </c>
       <c r="AG13" t="s" s="2">
-        <v>92</v>
+        <v>81</v>
       </c>
       <c r="AH13" t="s" s="2">
         <v>92</v>
       </c>
       <c r="AI13" t="s" s="2">
-        <v>80</v>
+        <v>178</v>
       </c>
       <c r="AJ13" t="s" s="2">
-        <v>80</v>
+        <v>104</v>
       </c>
       <c r="AK13" t="s" s="2">
-        <v>80</v>
+        <v>167</v>
       </c>
       <c r="AL13" t="s" s="2">
-        <v>80</v>
+        <v>179</v>
       </c>
       <c r="AM13" t="s" s="2">
-        <v>80</v>
+        <v>180</v>
       </c>
       <c r="AN13" t="s" s="2">
-        <v>135</v>
+        <v>181</v>
       </c>
       <c r="AO13" t="s" s="2">
-        <v>80</v>
+        <v>171</v>
       </c>
       <c r="AP13" t="s" s="2">
-        <v>80</v>
+        <v>182</v>
       </c>
     </row>
     <row r="14" hidden="true">
       <c r="A14" t="s" s="2">
-        <v>168</v>
+        <v>183</v>
       </c>
       <c r="B14" t="s" s="2">
-        <v>169</v>
+        <v>183</v>
       </c>
       <c r="C14" s="2"/>
       <c r="D14" t="s" s="2">
@@ -3136,10 +3205,10 @@
       </c>
       <c r="E14" s="2"/>
       <c r="F14" t="s" s="2">
-        <v>92</v>
+        <v>81</v>
       </c>
       <c r="G14" t="s" s="2">
-        <v>92</v>
+        <v>82</v>
       </c>
       <c r="H14" t="s" s="2">
         <v>80</v>
@@ -3151,15 +3220,17 @@
         <v>80</v>
       </c>
       <c r="K14" t="s" s="2">
-        <v>170</v>
+        <v>159</v>
       </c>
       <c r="L14" t="s" s="2">
-        <v>171</v>
+        <v>184</v>
       </c>
       <c r="M14" t="s" s="2">
-        <v>172</v>
-      </c>
-      <c r="N14" s="2"/>
+        <v>185</v>
+      </c>
+      <c r="N14" t="s" s="2">
+        <v>186</v>
+      </c>
       <c r="O14" s="2"/>
       <c r="P14" t="s" s="2">
         <v>80</v>
@@ -3184,13 +3255,13 @@
         <v>80</v>
       </c>
       <c r="X14" t="s" s="2">
-        <v>80</v>
+        <v>187</v>
       </c>
       <c r="Y14" t="s" s="2">
-        <v>80</v>
+        <v>185</v>
       </c>
       <c r="Z14" t="s" s="2">
-        <v>80</v>
+        <v>188</v>
       </c>
       <c r="AA14" t="s" s="2">
         <v>80</v>
@@ -3208,13 +3279,13 @@
         <v>80</v>
       </c>
       <c r="AF14" t="s" s="2">
-        <v>173</v>
+        <v>183</v>
       </c>
       <c r="AG14" t="s" s="2">
         <v>81</v>
       </c>
       <c r="AH14" t="s" s="2">
-        <v>92</v>
+        <v>82</v>
       </c>
       <c r="AI14" t="s" s="2">
         <v>80</v>
@@ -3226,16 +3297,16 @@
         <v>80</v>
       </c>
       <c r="AL14" t="s" s="2">
-        <v>80</v>
+        <v>189</v>
       </c>
       <c r="AM14" t="s" s="2">
-        <v>80</v>
+        <v>190</v>
       </c>
       <c r="AN14" t="s" s="2">
-        <v>135</v>
+        <v>191</v>
       </c>
       <c r="AO14" t="s" s="2">
-        <v>80</v>
+        <v>192</v>
       </c>
       <c r="AP14" t="s" s="2">
         <v>80</v>
@@ -3243,46 +3314,44 @@
     </row>
     <row r="15" hidden="true">
       <c r="A15" t="s" s="2">
-        <v>174</v>
+        <v>193</v>
       </c>
       <c r="B15" t="s" s="2">
-        <v>174</v>
+        <v>193</v>
       </c>
       <c r="C15" s="2"/>
       <c r="D15" t="s" s="2">
-        <v>175</v>
+        <v>80</v>
       </c>
       <c r="E15" s="2"/>
       <c r="F15" t="s" s="2">
         <v>81</v>
       </c>
       <c r="G15" t="s" s="2">
-        <v>82</v>
+        <v>92</v>
       </c>
       <c r="H15" t="s" s="2">
         <v>80</v>
       </c>
       <c r="I15" t="s" s="2">
-        <v>93</v>
+        <v>80</v>
       </c>
       <c r="J15" t="s" s="2">
         <v>80</v>
       </c>
       <c r="K15" t="s" s="2">
-        <v>137</v>
+        <v>159</v>
       </c>
       <c r="L15" t="s" s="2">
-        <v>176</v>
+        <v>194</v>
       </c>
       <c r="M15" t="s" s="2">
-        <v>177</v>
+        <v>195</v>
       </c>
       <c r="N15" t="s" s="2">
-        <v>178</v>
-      </c>
-      <c r="O15" t="s" s="2">
-        <v>179</v>
-      </c>
+        <v>196</v>
+      </c>
+      <c r="O15" s="2"/>
       <c r="P15" t="s" s="2">
         <v>80</v>
       </c>
@@ -3306,13 +3375,13 @@
         <v>80</v>
       </c>
       <c r="X15" t="s" s="2">
-        <v>80</v>
+        <v>116</v>
       </c>
       <c r="Y15" t="s" s="2">
-        <v>80</v>
+        <v>195</v>
       </c>
       <c r="Z15" t="s" s="2">
-        <v>80</v>
+        <v>197</v>
       </c>
       <c r="AA15" t="s" s="2">
         <v>80</v>
@@ -3330,59 +3399,59 @@
         <v>80</v>
       </c>
       <c r="AF15" t="s" s="2">
-        <v>180</v>
+        <v>193</v>
       </c>
       <c r="AG15" t="s" s="2">
         <v>81</v>
       </c>
       <c r="AH15" t="s" s="2">
-        <v>82</v>
+        <v>92</v>
       </c>
       <c r="AI15" t="s" s="2">
         <v>80</v>
       </c>
       <c r="AJ15" t="s" s="2">
-        <v>143</v>
+        <v>104</v>
       </c>
       <c r="AK15" t="s" s="2">
         <v>80</v>
       </c>
       <c r="AL15" t="s" s="2">
-        <v>80</v>
+        <v>198</v>
       </c>
       <c r="AM15" t="s" s="2">
-        <v>80</v>
+        <v>199</v>
       </c>
       <c r="AN15" t="s" s="2">
-        <v>135</v>
+        <v>200</v>
       </c>
       <c r="AO15" t="s" s="2">
-        <v>80</v>
+        <v>201</v>
       </c>
       <c r="AP15" t="s" s="2">
-        <v>80</v>
+        <v>202</v>
       </c>
     </row>
-    <row r="16" hidden="true">
+    <row r="16">
       <c r="A16" t="s" s="2">
-        <v>181</v>
+        <v>203</v>
       </c>
       <c r="B16" t="s" s="2">
-        <v>181</v>
+        <v>203</v>
       </c>
       <c r="C16" s="2"/>
       <c r="D16" t="s" s="2">
-        <v>80</v>
+        <v>204</v>
       </c>
       <c r="E16" s="2"/>
       <c r="F16" t="s" s="2">
-        <v>81</v>
+        <v>92</v>
       </c>
       <c r="G16" t="s" s="2">
-        <v>82</v>
+        <v>92</v>
       </c>
       <c r="H16" t="s" s="2">
-        <v>80</v>
+        <v>93</v>
       </c>
       <c r="I16" t="s" s="2">
         <v>80</v>
@@ -3391,19 +3460,17 @@
         <v>93</v>
       </c>
       <c r="K16" t="s" s="2">
-        <v>182</v>
+        <v>159</v>
       </c>
       <c r="L16" t="s" s="2">
-        <v>183</v>
+        <v>205</v>
       </c>
       <c r="M16" t="s" s="2">
-        <v>184</v>
-      </c>
-      <c r="N16" t="s" s="2">
-        <v>185</v>
-      </c>
+        <v>206</v>
+      </c>
+      <c r="N16" s="2"/>
       <c r="O16" t="s" s="2">
-        <v>186</v>
+        <v>207</v>
       </c>
       <c r="P16" t="s" s="2">
         <v>80</v>
@@ -3428,13 +3495,13 @@
         <v>80</v>
       </c>
       <c r="X16" t="s" s="2">
-        <v>80</v>
+        <v>208</v>
       </c>
       <c r="Y16" t="s" s="2">
-        <v>80</v>
+        <v>209</v>
       </c>
       <c r="Z16" t="s" s="2">
-        <v>80</v>
+        <v>210</v>
       </c>
       <c r="AA16" t="s" s="2">
         <v>80</v>
@@ -3452,13 +3519,13 @@
         <v>80</v>
       </c>
       <c r="AF16" t="s" s="2">
-        <v>181</v>
+        <v>203</v>
       </c>
       <c r="AG16" t="s" s="2">
         <v>81</v>
       </c>
       <c r="AH16" t="s" s="2">
-        <v>82</v>
+        <v>92</v>
       </c>
       <c r="AI16" t="s" s="2">
         <v>80</v>
@@ -3467,30 +3534,30 @@
         <v>104</v>
       </c>
       <c r="AK16" t="s" s="2">
-        <v>187</v>
+        <v>211</v>
       </c>
       <c r="AL16" t="s" s="2">
-        <v>80</v>
+        <v>212</v>
       </c>
       <c r="AM16" t="s" s="2">
-        <v>80</v>
+        <v>213</v>
       </c>
       <c r="AN16" t="s" s="2">
-        <v>188</v>
+        <v>214</v>
       </c>
       <c r="AO16" t="s" s="2">
-        <v>189</v>
+        <v>215</v>
       </c>
       <c r="AP16" t="s" s="2">
-        <v>80</v>
+        <v>216</v>
       </c>
     </row>
-    <row r="17" hidden="true">
+    <row r="17">
       <c r="A17" t="s" s="2">
-        <v>190</v>
+        <v>217</v>
       </c>
       <c r="B17" t="s" s="2">
-        <v>190</v>
+        <v>217</v>
       </c>
       <c r="C17" s="2"/>
       <c r="D17" t="s" s="2">
@@ -3501,28 +3568,28 @@
         <v>81</v>
       </c>
       <c r="G17" t="s" s="2">
-        <v>92</v>
+        <v>82</v>
       </c>
       <c r="H17" t="s" s="2">
-        <v>80</v>
+        <v>93</v>
       </c>
       <c r="I17" t="s" s="2">
-        <v>93</v>
+        <v>80</v>
       </c>
       <c r="J17" t="s" s="2">
         <v>93</v>
       </c>
       <c r="K17" t="s" s="2">
-        <v>191</v>
+        <v>159</v>
       </c>
       <c r="L17" t="s" s="2">
-        <v>192</v>
+        <v>218</v>
       </c>
       <c r="M17" t="s" s="2">
-        <v>193</v>
+        <v>219</v>
       </c>
       <c r="N17" t="s" s="2">
-        <v>194</v>
+        <v>220</v>
       </c>
       <c r="O17" s="2"/>
       <c r="P17" t="s" s="2">
@@ -3548,13 +3615,13 @@
         <v>80</v>
       </c>
       <c r="X17" t="s" s="2">
-        <v>195</v>
+        <v>208</v>
       </c>
       <c r="Y17" t="s" s="2">
-        <v>196</v>
+        <v>221</v>
       </c>
       <c r="Z17" t="s" s="2">
-        <v>197</v>
+        <v>222</v>
       </c>
       <c r="AA17" t="s" s="2">
         <v>80</v>
@@ -3572,45 +3639,45 @@
         <v>80</v>
       </c>
       <c r="AF17" t="s" s="2">
-        <v>190</v>
+        <v>217</v>
       </c>
       <c r="AG17" t="s" s="2">
         <v>81</v>
       </c>
       <c r="AH17" t="s" s="2">
-        <v>92</v>
+        <v>82</v>
       </c>
       <c r="AI17" t="s" s="2">
-        <v>198</v>
+        <v>80</v>
       </c>
       <c r="AJ17" t="s" s="2">
         <v>104</v>
       </c>
       <c r="AK17" t="s" s="2">
-        <v>199</v>
+        <v>80</v>
       </c>
       <c r="AL17" t="s" s="2">
-        <v>200</v>
+        <v>223</v>
       </c>
       <c r="AM17" t="s" s="2">
-        <v>201</v>
+        <v>80</v>
       </c>
       <c r="AN17" t="s" s="2">
-        <v>202</v>
+        <v>224</v>
       </c>
       <c r="AO17" t="s" s="2">
-        <v>203</v>
+        <v>80</v>
       </c>
       <c r="AP17" t="s" s="2">
-        <v>80</v>
+        <v>225</v>
       </c>
     </row>
     <row r="18" hidden="true">
       <c r="A18" t="s" s="2">
-        <v>204</v>
+        <v>226</v>
       </c>
       <c r="B18" t="s" s="2">
-        <v>204</v>
+        <v>226</v>
       </c>
       <c r="C18" s="2"/>
       <c r="D18" t="s" s="2">
@@ -3627,23 +3694,21 @@
         <v>80</v>
       </c>
       <c r="I18" t="s" s="2">
-        <v>93</v>
+        <v>80</v>
       </c>
       <c r="J18" t="s" s="2">
-        <v>93</v>
+        <v>80</v>
       </c>
       <c r="K18" t="s" s="2">
-        <v>191</v>
+        <v>227</v>
       </c>
       <c r="L18" t="s" s="2">
-        <v>205</v>
+        <v>228</v>
       </c>
       <c r="M18" t="s" s="2">
-        <v>206</v>
-      </c>
-      <c r="N18" t="s" s="2">
-        <v>207</v>
-      </c>
+        <v>229</v>
+      </c>
+      <c r="N18" s="2"/>
       <c r="O18" s="2"/>
       <c r="P18" t="s" s="2">
         <v>80</v>
@@ -3668,13 +3733,13 @@
         <v>80</v>
       </c>
       <c r="X18" t="s" s="2">
-        <v>195</v>
+        <v>80</v>
       </c>
       <c r="Y18" t="s" s="2">
-        <v>208</v>
+        <v>80</v>
       </c>
       <c r="Z18" t="s" s="2">
-        <v>209</v>
+        <v>80</v>
       </c>
       <c r="AA18" t="s" s="2">
         <v>80</v>
@@ -3692,7 +3757,7 @@
         <v>80</v>
       </c>
       <c r="AF18" t="s" s="2">
-        <v>204</v>
+        <v>230</v>
       </c>
       <c r="AG18" t="s" s="2">
         <v>81</v>
@@ -3701,40 +3766,40 @@
         <v>92</v>
       </c>
       <c r="AI18" t="s" s="2">
-        <v>210</v>
+        <v>80</v>
       </c>
       <c r="AJ18" t="s" s="2">
-        <v>104</v>
+        <v>80</v>
       </c>
       <c r="AK18" t="s" s="2">
-        <v>199</v>
+        <v>80</v>
       </c>
       <c r="AL18" t="s" s="2">
-        <v>211</v>
+        <v>80</v>
       </c>
       <c r="AM18" t="s" s="2">
-        <v>212</v>
+        <v>80</v>
       </c>
       <c r="AN18" t="s" s="2">
-        <v>213</v>
+        <v>231</v>
       </c>
       <c r="AO18" t="s" s="2">
-        <v>203</v>
+        <v>80</v>
       </c>
       <c r="AP18" t="s" s="2">
-        <v>214</v>
+        <v>80</v>
       </c>
     </row>
     <row r="19" hidden="true">
       <c r="A19" t="s" s="2">
-        <v>215</v>
+        <v>232</v>
       </c>
       <c r="B19" t="s" s="2">
-        <v>215</v>
+        <v>232</v>
       </c>
       <c r="C19" s="2"/>
       <c r="D19" t="s" s="2">
-        <v>80</v>
+        <v>137</v>
       </c>
       <c r="E19" s="2"/>
       <c r="F19" t="s" s="2">
@@ -3753,16 +3818,16 @@
         <v>80</v>
       </c>
       <c r="K19" t="s" s="2">
-        <v>191</v>
+        <v>138</v>
       </c>
       <c r="L19" t="s" s="2">
-        <v>216</v>
+        <v>139</v>
       </c>
       <c r="M19" t="s" s="2">
-        <v>217</v>
+        <v>233</v>
       </c>
       <c r="N19" t="s" s="2">
-        <v>218</v>
+        <v>141</v>
       </c>
       <c r="O19" s="2"/>
       <c r="P19" t="s" s="2">
@@ -3788,31 +3853,31 @@
         <v>80</v>
       </c>
       <c r="X19" t="s" s="2">
-        <v>219</v>
+        <v>80</v>
       </c>
       <c r="Y19" t="s" s="2">
-        <v>217</v>
+        <v>80</v>
       </c>
       <c r="Z19" t="s" s="2">
-        <v>220</v>
+        <v>80</v>
       </c>
       <c r="AA19" t="s" s="2">
         <v>80</v>
       </c>
       <c r="AB19" t="s" s="2">
-        <v>80</v>
+        <v>234</v>
       </c>
       <c r="AC19" t="s" s="2">
-        <v>80</v>
+        <v>235</v>
       </c>
       <c r="AD19" t="s" s="2">
         <v>80</v>
       </c>
       <c r="AE19" t="s" s="2">
-        <v>80</v>
+        <v>236</v>
       </c>
       <c r="AF19" t="s" s="2">
-        <v>215</v>
+        <v>237</v>
       </c>
       <c r="AG19" t="s" s="2">
         <v>81</v>
@@ -3824,35 +3889,37 @@
         <v>80</v>
       </c>
       <c r="AJ19" t="s" s="2">
-        <v>104</v>
+        <v>143</v>
       </c>
       <c r="AK19" t="s" s="2">
         <v>80</v>
       </c>
       <c r="AL19" t="s" s="2">
-        <v>221</v>
+        <v>80</v>
       </c>
       <c r="AM19" t="s" s="2">
-        <v>222</v>
+        <v>80</v>
       </c>
       <c r="AN19" t="s" s="2">
-        <v>223</v>
+        <v>231</v>
       </c>
       <c r="AO19" t="s" s="2">
-        <v>224</v>
+        <v>80</v>
       </c>
       <c r="AP19" t="s" s="2">
         <v>80</v>
       </c>
     </row>
-    <row r="20" hidden="true">
+    <row r="20">
       <c r="A20" t="s" s="2">
-        <v>225</v>
+        <v>238</v>
       </c>
       <c r="B20" t="s" s="2">
-        <v>225</v>
-      </c>
-      <c r="C20" s="2"/>
+        <v>232</v>
+      </c>
+      <c r="C20" t="s" s="2">
+        <v>239</v>
+      </c>
       <c r="D20" t="s" s="2">
         <v>80</v>
       </c>
@@ -3864,7 +3931,7 @@
         <v>92</v>
       </c>
       <c r="H20" t="s" s="2">
-        <v>80</v>
+        <v>93</v>
       </c>
       <c r="I20" t="s" s="2">
         <v>80</v>
@@ -3873,17 +3940,15 @@
         <v>80</v>
       </c>
       <c r="K20" t="s" s="2">
-        <v>191</v>
+        <v>240</v>
       </c>
       <c r="L20" t="s" s="2">
-        <v>226</v>
+        <v>241</v>
       </c>
       <c r="M20" t="s" s="2">
-        <v>227</v>
-      </c>
-      <c r="N20" t="s" s="2">
-        <v>228</v>
-      </c>
+        <v>242</v>
+      </c>
+      <c r="N20" s="2"/>
       <c r="O20" s="2"/>
       <c r="P20" t="s" s="2">
         <v>80</v>
@@ -3908,13 +3973,13 @@
         <v>80</v>
       </c>
       <c r="X20" t="s" s="2">
-        <v>116</v>
+        <v>80</v>
       </c>
       <c r="Y20" t="s" s="2">
-        <v>227</v>
+        <v>80</v>
       </c>
       <c r="Z20" t="s" s="2">
-        <v>229</v>
+        <v>80</v>
       </c>
       <c r="AA20" t="s" s="2">
         <v>80</v>
@@ -3932,79 +3997,77 @@
         <v>80</v>
       </c>
       <c r="AF20" t="s" s="2">
-        <v>225</v>
+        <v>237</v>
       </c>
       <c r="AG20" t="s" s="2">
         <v>81</v>
       </c>
       <c r="AH20" t="s" s="2">
-        <v>92</v>
+        <v>82</v>
       </c>
       <c r="AI20" t="s" s="2">
         <v>80</v>
       </c>
       <c r="AJ20" t="s" s="2">
-        <v>104</v>
+        <v>143</v>
       </c>
       <c r="AK20" t="s" s="2">
         <v>80</v>
       </c>
       <c r="AL20" t="s" s="2">
-        <v>230</v>
+        <v>80</v>
       </c>
       <c r="AM20" t="s" s="2">
-        <v>231</v>
+        <v>80</v>
       </c>
       <c r="AN20" t="s" s="2">
-        <v>232</v>
+        <v>80</v>
       </c>
       <c r="AO20" t="s" s="2">
-        <v>233</v>
+        <v>80</v>
       </c>
       <c r="AP20" t="s" s="2">
-        <v>234</v>
+        <v>80</v>
       </c>
     </row>
-    <row r="21">
+    <row r="21" hidden="true">
       <c r="A21" t="s" s="2">
-        <v>235</v>
+        <v>243</v>
       </c>
       <c r="B21" t="s" s="2">
-        <v>235</v>
+        <v>244</v>
       </c>
       <c r="C21" s="2"/>
       <c r="D21" t="s" s="2">
-        <v>236</v>
+        <v>80</v>
       </c>
       <c r="E21" s="2"/>
       <c r="F21" t="s" s="2">
-        <v>92</v>
+        <v>81</v>
       </c>
       <c r="G21" t="s" s="2">
         <v>92</v>
       </c>
       <c r="H21" t="s" s="2">
-        <v>93</v>
+        <v>80</v>
       </c>
       <c r="I21" t="s" s="2">
         <v>80</v>
       </c>
       <c r="J21" t="s" s="2">
-        <v>93</v>
+        <v>80</v>
       </c>
       <c r="K21" t="s" s="2">
-        <v>191</v>
+        <v>227</v>
       </c>
       <c r="L21" t="s" s="2">
-        <v>237</v>
+        <v>228</v>
       </c>
       <c r="M21" t="s" s="2">
-        <v>238</v>
+        <v>229</v>
       </c>
       <c r="N21" s="2"/>
-      <c r="O21" t="s" s="2">
-        <v>239</v>
-      </c>
+      <c r="O21" s="2"/>
       <c r="P21" t="s" s="2">
         <v>80</v>
       </c>
@@ -4028,13 +4091,13 @@
         <v>80</v>
       </c>
       <c r="X21" t="s" s="2">
-        <v>240</v>
+        <v>80</v>
       </c>
       <c r="Y21" t="s" s="2">
-        <v>241</v>
+        <v>80</v>
       </c>
       <c r="Z21" t="s" s="2">
-        <v>242</v>
+        <v>80</v>
       </c>
       <c r="AA21" t="s" s="2">
         <v>80</v>
@@ -4052,7 +4115,7 @@
         <v>80</v>
       </c>
       <c r="AF21" t="s" s="2">
-        <v>235</v>
+        <v>230</v>
       </c>
       <c r="AG21" t="s" s="2">
         <v>81</v>
@@ -4064,33 +4127,33 @@
         <v>80</v>
       </c>
       <c r="AJ21" t="s" s="2">
-        <v>104</v>
+        <v>80</v>
       </c>
       <c r="AK21" t="s" s="2">
-        <v>243</v>
+        <v>80</v>
       </c>
       <c r="AL21" t="s" s="2">
-        <v>244</v>
+        <v>80</v>
       </c>
       <c r="AM21" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="AN21" t="s" s="2">
+        <v>231</v>
+      </c>
+      <c r="AO21" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="AP21" t="s" s="2">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="22" hidden="true">
+      <c r="A22" t="s" s="2">
         <v>245</v>
       </c>
-      <c r="AN21" t="s" s="2">
+      <c r="B22" t="s" s="2">
         <v>246</v>
-      </c>
-      <c r="AO21" t="s" s="2">
-        <v>247</v>
-      </c>
-      <c r="AP21" t="s" s="2">
-        <v>248</v>
-      </c>
-    </row>
-    <row r="22">
-      <c r="A22" t="s" s="2">
-        <v>249</v>
-      </c>
-      <c r="B22" t="s" s="2">
-        <v>249</v>
       </c>
       <c r="C22" s="2"/>
       <c r="D22" t="s" s="2">
@@ -4101,29 +4164,27 @@
         <v>81</v>
       </c>
       <c r="G22" t="s" s="2">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="H22" t="s" s="2">
-        <v>93</v>
+        <v>80</v>
       </c>
       <c r="I22" t="s" s="2">
         <v>80</v>
       </c>
       <c r="J22" t="s" s="2">
-        <v>93</v>
+        <v>80</v>
       </c>
       <c r="K22" t="s" s="2">
-        <v>191</v>
+        <v>138</v>
       </c>
       <c r="L22" t="s" s="2">
-        <v>250</v>
+        <v>247</v>
       </c>
       <c r="M22" t="s" s="2">
-        <v>251</v>
-      </c>
-      <c r="N22" t="s" s="2">
-        <v>252</v>
-      </c>
+        <v>248</v>
+      </c>
+      <c r="N22" s="2"/>
       <c r="O22" s="2"/>
       <c r="P22" t="s" s="2">
         <v>80</v>
@@ -4148,31 +4209,31 @@
         <v>80</v>
       </c>
       <c r="X22" t="s" s="2">
-        <v>240</v>
+        <v>80</v>
       </c>
       <c r="Y22" t="s" s="2">
-        <v>253</v>
+        <v>80</v>
       </c>
       <c r="Z22" t="s" s="2">
-        <v>254</v>
+        <v>80</v>
       </c>
       <c r="AA22" t="s" s="2">
         <v>80</v>
       </c>
       <c r="AB22" t="s" s="2">
-        <v>80</v>
+        <v>234</v>
       </c>
       <c r="AC22" t="s" s="2">
-        <v>80</v>
+        <v>235</v>
       </c>
       <c r="AD22" t="s" s="2">
         <v>80</v>
       </c>
       <c r="AE22" t="s" s="2">
-        <v>80</v>
+        <v>236</v>
       </c>
       <c r="AF22" t="s" s="2">
-        <v>249</v>
+        <v>237</v>
       </c>
       <c r="AG22" t="s" s="2">
         <v>81</v>
@@ -4184,37 +4245,37 @@
         <v>80</v>
       </c>
       <c r="AJ22" t="s" s="2">
-        <v>104</v>
+        <v>143</v>
       </c>
       <c r="AK22" t="s" s="2">
         <v>80</v>
       </c>
       <c r="AL22" t="s" s="2">
-        <v>255</v>
+        <v>80</v>
       </c>
       <c r="AM22" t="s" s="2">
         <v>80</v>
       </c>
       <c r="AN22" t="s" s="2">
-        <v>256</v>
+        <v>80</v>
       </c>
       <c r="AO22" t="s" s="2">
         <v>80</v>
       </c>
       <c r="AP22" t="s" s="2">
-        <v>257</v>
+        <v>80</v>
       </c>
     </row>
-    <row r="23">
+    <row r="23" hidden="true">
       <c r="A23" t="s" s="2">
-        <v>258</v>
+        <v>249</v>
       </c>
       <c r="B23" t="s" s="2">
-        <v>258</v>
+        <v>250</v>
       </c>
       <c r="C23" s="2"/>
       <c r="D23" t="s" s="2">
-        <v>259</v>
+        <v>80</v>
       </c>
       <c r="E23" s="2"/>
       <c r="F23" t="s" s="2">
@@ -4224,33 +4285,33 @@
         <v>92</v>
       </c>
       <c r="H23" t="s" s="2">
-        <v>93</v>
+        <v>80</v>
       </c>
       <c r="I23" t="s" s="2">
         <v>80</v>
       </c>
       <c r="J23" t="s" s="2">
-        <v>93</v>
+        <v>80</v>
       </c>
       <c r="K23" t="s" s="2">
-        <v>260</v>
+        <v>106</v>
       </c>
       <c r="L23" t="s" s="2">
-        <v>261</v>
+        <v>251</v>
       </c>
       <c r="M23" t="s" s="2">
-        <v>262</v>
-      </c>
-      <c r="N23" s="2"/>
-      <c r="O23" t="s" s="2">
-        <v>263</v>
-      </c>
+        <v>252</v>
+      </c>
+      <c r="N23" t="s" s="2">
+        <v>253</v>
+      </c>
+      <c r="O23" s="2"/>
       <c r="P23" t="s" s="2">
         <v>80</v>
       </c>
       <c r="Q23" s="2"/>
       <c r="R23" t="s" s="2">
-        <v>80</v>
+        <v>254</v>
       </c>
       <c r="S23" t="s" s="2">
         <v>80</v>
@@ -4292,7 +4353,7 @@
         <v>80</v>
       </c>
       <c r="AF23" t="s" s="2">
-        <v>258</v>
+        <v>255</v>
       </c>
       <c r="AG23" t="s" s="2">
         <v>92</v>
@@ -4304,22 +4365,22 @@
         <v>80</v>
       </c>
       <c r="AJ23" t="s" s="2">
-        <v>104</v>
+        <v>80</v>
       </c>
       <c r="AK23" t="s" s="2">
-        <v>264</v>
+        <v>80</v>
       </c>
       <c r="AL23" t="s" s="2">
         <v>80</v>
       </c>
       <c r="AM23" t="s" s="2">
-        <v>265</v>
+        <v>80</v>
       </c>
       <c r="AN23" t="s" s="2">
-        <v>266</v>
+        <v>135</v>
       </c>
       <c r="AO23" t="s" s="2">
-        <v>267</v>
+        <v>80</v>
       </c>
       <c r="AP23" t="s" s="2">
         <v>80</v>
@@ -4327,10 +4388,10 @@
     </row>
     <row r="24" hidden="true">
       <c r="A24" t="s" s="2">
-        <v>268</v>
+        <v>256</v>
       </c>
       <c r="B24" t="s" s="2">
-        <v>268</v>
+        <v>257</v>
       </c>
       <c r="C24" s="2"/>
       <c r="D24" t="s" s="2">
@@ -4338,7 +4399,7 @@
       </c>
       <c r="E24" s="2"/>
       <c r="F24" t="s" s="2">
-        <v>81</v>
+        <v>92</v>
       </c>
       <c r="G24" t="s" s="2">
         <v>92</v>
@@ -4350,20 +4411,18 @@
         <v>80</v>
       </c>
       <c r="J24" t="s" s="2">
-        <v>93</v>
+        <v>80</v>
       </c>
       <c r="K24" t="s" s="2">
-        <v>269</v>
+        <v>258</v>
       </c>
       <c r="L24" t="s" s="2">
-        <v>270</v>
+        <v>259</v>
       </c>
       <c r="M24" t="s" s="2">
-        <v>271</v>
-      </c>
-      <c r="N24" t="s" s="2">
-        <v>272</v>
-      </c>
+        <v>260</v>
+      </c>
+      <c r="N24" s="2"/>
       <c r="O24" s="2"/>
       <c r="P24" t="s" s="2">
         <v>80</v>
@@ -4412,7 +4471,7 @@
         <v>80</v>
       </c>
       <c r="AF24" t="s" s="2">
-        <v>268</v>
+        <v>261</v>
       </c>
       <c r="AG24" t="s" s="2">
         <v>81</v>
@@ -4427,19 +4486,19 @@
         <v>104</v>
       </c>
       <c r="AK24" t="s" s="2">
-        <v>273</v>
+        <v>80</v>
       </c>
       <c r="AL24" t="s" s="2">
         <v>80</v>
       </c>
       <c r="AM24" t="s" s="2">
-        <v>274</v>
+        <v>80</v>
       </c>
       <c r="AN24" t="s" s="2">
-        <v>275</v>
+        <v>135</v>
       </c>
       <c r="AO24" t="s" s="2">
-        <v>276</v>
+        <v>80</v>
       </c>
       <c r="AP24" t="s" s="2">
         <v>80</v>
@@ -4447,10 +4506,10 @@
     </row>
     <row r="25" hidden="true">
       <c r="A25" t="s" s="2">
-        <v>277</v>
+        <v>262</v>
       </c>
       <c r="B25" t="s" s="2">
-        <v>277</v>
+        <v>262</v>
       </c>
       <c r="C25" s="2"/>
       <c r="D25" t="s" s="2">
@@ -4461,7 +4520,7 @@
         <v>81</v>
       </c>
       <c r="G25" t="s" s="2">
-        <v>92</v>
+        <v>82</v>
       </c>
       <c r="H25" t="s" s="2">
         <v>80</v>
@@ -4473,18 +4532,20 @@
         <v>93</v>
       </c>
       <c r="K25" t="s" s="2">
-        <v>278</v>
+        <v>263</v>
       </c>
       <c r="L25" t="s" s="2">
-        <v>279</v>
+        <v>264</v>
       </c>
       <c r="M25" t="s" s="2">
-        <v>280</v>
+        <v>265</v>
       </c>
       <c r="N25" t="s" s="2">
-        <v>281</v>
-      </c>
-      <c r="O25" s="2"/>
+        <v>266</v>
+      </c>
+      <c r="O25" t="s" s="2">
+        <v>267</v>
+      </c>
       <c r="P25" t="s" s="2">
         <v>80</v>
       </c>
@@ -4532,13 +4593,13 @@
         <v>80</v>
       </c>
       <c r="AF25" t="s" s="2">
-        <v>277</v>
+        <v>268</v>
       </c>
       <c r="AG25" t="s" s="2">
         <v>81</v>
       </c>
       <c r="AH25" t="s" s="2">
-        <v>92</v>
+        <v>82</v>
       </c>
       <c r="AI25" t="s" s="2">
         <v>80</v>
@@ -4547,19 +4608,19 @@
         <v>104</v>
       </c>
       <c r="AK25" t="s" s="2">
-        <v>282</v>
+        <v>80</v>
       </c>
       <c r="AL25" t="s" s="2">
         <v>80</v>
       </c>
       <c r="AM25" t="s" s="2">
-        <v>283</v>
+        <v>269</v>
       </c>
       <c r="AN25" t="s" s="2">
-        <v>284</v>
+        <v>270</v>
       </c>
       <c r="AO25" t="s" s="2">
-        <v>285</v>
+        <v>80</v>
       </c>
       <c r="AP25" t="s" s="2">
         <v>80</v>
@@ -4567,10 +4628,10 @@
     </row>
     <row r="26" hidden="true">
       <c r="A26" t="s" s="2">
-        <v>286</v>
+        <v>271</v>
       </c>
       <c r="B26" t="s" s="2">
-        <v>286</v>
+        <v>271</v>
       </c>
       <c r="C26" s="2"/>
       <c r="D26" t="s" s="2">
@@ -4590,21 +4651,23 @@
         <v>80</v>
       </c>
       <c r="J26" t="s" s="2">
-        <v>80</v>
+        <v>93</v>
       </c>
       <c r="K26" t="s" s="2">
-        <v>278</v>
+        <v>227</v>
       </c>
       <c r="L26" t="s" s="2">
-        <v>287</v>
+        <v>272</v>
       </c>
       <c r="M26" t="s" s="2">
-        <v>288</v>
+        <v>273</v>
       </c>
       <c r="N26" t="s" s="2">
-        <v>289</v>
-      </c>
-      <c r="O26" s="2"/>
+        <v>274</v>
+      </c>
+      <c r="O26" t="s" s="2">
+        <v>275</v>
+      </c>
       <c r="P26" t="s" s="2">
         <v>80</v>
       </c>
@@ -4652,7 +4715,7 @@
         <v>80</v>
       </c>
       <c r="AF26" t="s" s="2">
-        <v>286</v>
+        <v>276</v>
       </c>
       <c r="AG26" t="s" s="2">
         <v>81</v>
@@ -4661,7 +4724,7 @@
         <v>92</v>
       </c>
       <c r="AI26" t="s" s="2">
-        <v>290</v>
+        <v>80</v>
       </c>
       <c r="AJ26" t="s" s="2">
         <v>104</v>
@@ -4673,38 +4736,38 @@
         <v>80</v>
       </c>
       <c r="AM26" t="s" s="2">
-        <v>80</v>
+        <v>277</v>
       </c>
       <c r="AN26" t="s" s="2">
-        <v>291</v>
+        <v>278</v>
       </c>
       <c r="AO26" t="s" s="2">
-        <v>292</v>
+        <v>80</v>
       </c>
       <c r="AP26" t="s" s="2">
         <v>80</v>
       </c>
     </row>
-    <row r="27" hidden="true">
+    <row r="27">
       <c r="A27" t="s" s="2">
-        <v>293</v>
+        <v>279</v>
       </c>
       <c r="B27" t="s" s="2">
-        <v>293</v>
+        <v>279</v>
       </c>
       <c r="C27" s="2"/>
       <c r="D27" t="s" s="2">
-        <v>80</v>
+        <v>280</v>
       </c>
       <c r="E27" s="2"/>
       <c r="F27" t="s" s="2">
-        <v>81</v>
+        <v>92</v>
       </c>
       <c r="G27" t="s" s="2">
         <v>92</v>
       </c>
       <c r="H27" t="s" s="2">
-        <v>80</v>
+        <v>93</v>
       </c>
       <c r="I27" t="s" s="2">
         <v>80</v>
@@ -4713,16 +4776,18 @@
         <v>93</v>
       </c>
       <c r="K27" t="s" s="2">
-        <v>294</v>
+        <v>281</v>
       </c>
       <c r="L27" t="s" s="2">
-        <v>295</v>
+        <v>282</v>
       </c>
       <c r="M27" t="s" s="2">
-        <v>296</v>
+        <v>283</v>
       </c>
       <c r="N27" s="2"/>
-      <c r="O27" s="2"/>
+      <c r="O27" t="s" s="2">
+        <v>284</v>
+      </c>
       <c r="P27" t="s" s="2">
         <v>80</v>
       </c>
@@ -4770,10 +4835,10 @@
         <v>80</v>
       </c>
       <c r="AF27" t="s" s="2">
-        <v>293</v>
+        <v>279</v>
       </c>
       <c r="AG27" t="s" s="2">
-        <v>81</v>
+        <v>92</v>
       </c>
       <c r="AH27" t="s" s="2">
         <v>92</v>
@@ -4785,19 +4850,19 @@
         <v>104</v>
       </c>
       <c r="AK27" t="s" s="2">
-        <v>80</v>
+        <v>285</v>
       </c>
       <c r="AL27" t="s" s="2">
         <v>80</v>
       </c>
       <c r="AM27" t="s" s="2">
-        <v>297</v>
+        <v>286</v>
       </c>
       <c r="AN27" t="s" s="2">
-        <v>298</v>
+        <v>287</v>
       </c>
       <c r="AO27" t="s" s="2">
-        <v>299</v>
+        <v>288</v>
       </c>
       <c r="AP27" t="s" s="2">
         <v>80</v>
@@ -4805,10 +4870,10 @@
     </row>
     <row r="28" hidden="true">
       <c r="A28" t="s" s="2">
-        <v>300</v>
+        <v>289</v>
       </c>
       <c r="B28" t="s" s="2">
-        <v>300</v>
+        <v>289</v>
       </c>
       <c r="C28" s="2"/>
       <c r="D28" t="s" s="2">
@@ -4831,15 +4896,17 @@
         <v>93</v>
       </c>
       <c r="K28" t="s" s="2">
-        <v>301</v>
+        <v>290</v>
       </c>
       <c r="L28" t="s" s="2">
-        <v>302</v>
+        <v>291</v>
       </c>
       <c r="M28" t="s" s="2">
-        <v>303</v>
-      </c>
-      <c r="N28" s="2"/>
+        <v>292</v>
+      </c>
+      <c r="N28" t="s" s="2">
+        <v>293</v>
+      </c>
       <c r="O28" s="2"/>
       <c r="P28" t="s" s="2">
         <v>80</v>
@@ -4888,7 +4955,7 @@
         <v>80</v>
       </c>
       <c r="AF28" t="s" s="2">
-        <v>300</v>
+        <v>289</v>
       </c>
       <c r="AG28" t="s" s="2">
         <v>81</v>
@@ -4903,19 +4970,19 @@
         <v>104</v>
       </c>
       <c r="AK28" t="s" s="2">
-        <v>80</v>
+        <v>294</v>
       </c>
       <c r="AL28" t="s" s="2">
         <v>80</v>
       </c>
       <c r="AM28" t="s" s="2">
-        <v>80</v>
+        <v>295</v>
       </c>
       <c r="AN28" t="s" s="2">
-        <v>304</v>
+        <v>296</v>
       </c>
       <c r="AO28" t="s" s="2">
-        <v>305</v>
+        <v>297</v>
       </c>
       <c r="AP28" t="s" s="2">
         <v>80</v>
@@ -4923,10 +4990,10 @@
     </row>
     <row r="29" hidden="true">
       <c r="A29" t="s" s="2">
-        <v>306</v>
+        <v>298</v>
       </c>
       <c r="B29" t="s" s="2">
-        <v>306</v>
+        <v>298</v>
       </c>
       <c r="C29" s="2"/>
       <c r="D29" t="s" s="2">
@@ -4949,15 +5016,17 @@
         <v>93</v>
       </c>
       <c r="K29" t="s" s="2">
+        <v>299</v>
+      </c>
+      <c r="L29" t="s" s="2">
+        <v>300</v>
+      </c>
+      <c r="M29" t="s" s="2">
         <v>301</v>
       </c>
-      <c r="L29" t="s" s="2">
-        <v>307</v>
-      </c>
-      <c r="M29" t="s" s="2">
-        <v>308</v>
-      </c>
-      <c r="N29" s="2"/>
+      <c r="N29" t="s" s="2">
+        <v>302</v>
+      </c>
       <c r="O29" s="2"/>
       <c r="P29" t="s" s="2">
         <v>80</v>
@@ -5006,7 +5075,7 @@
         <v>80</v>
       </c>
       <c r="AF29" t="s" s="2">
-        <v>306</v>
+        <v>298</v>
       </c>
       <c r="AG29" t="s" s="2">
         <v>81</v>
@@ -5021,19 +5090,19 @@
         <v>104</v>
       </c>
       <c r="AK29" t="s" s="2">
-        <v>80</v>
+        <v>303</v>
       </c>
       <c r="AL29" t="s" s="2">
         <v>80</v>
       </c>
       <c r="AM29" t="s" s="2">
-        <v>309</v>
+        <v>304</v>
       </c>
       <c r="AN29" t="s" s="2">
-        <v>310</v>
+        <v>305</v>
       </c>
       <c r="AO29" t="s" s="2">
-        <v>311</v>
+        <v>306</v>
       </c>
       <c r="AP29" t="s" s="2">
         <v>80</v>
@@ -5041,10 +5110,10 @@
     </row>
     <row r="30" hidden="true">
       <c r="A30" t="s" s="2">
-        <v>312</v>
+        <v>307</v>
       </c>
       <c r="B30" t="s" s="2">
-        <v>312</v>
+        <v>307</v>
       </c>
       <c r="C30" s="2"/>
       <c r="D30" t="s" s="2">
@@ -5055,7 +5124,7 @@
         <v>81</v>
       </c>
       <c r="G30" t="s" s="2">
-        <v>82</v>
+        <v>92</v>
       </c>
       <c r="H30" t="s" s="2">
         <v>80</v>
@@ -5067,15 +5136,17 @@
         <v>80</v>
       </c>
       <c r="K30" t="s" s="2">
-        <v>313</v>
+        <v>299</v>
       </c>
       <c r="L30" t="s" s="2">
-        <v>314</v>
+        <v>308</v>
       </c>
       <c r="M30" t="s" s="2">
-        <v>315</v>
-      </c>
-      <c r="N30" s="2"/>
+        <v>309</v>
+      </c>
+      <c r="N30" t="s" s="2">
+        <v>310</v>
+      </c>
       <c r="O30" s="2"/>
       <c r="P30" t="s" s="2">
         <v>80</v>
@@ -5124,34 +5195,34 @@
         <v>80</v>
       </c>
       <c r="AF30" t="s" s="2">
+        <v>307</v>
+      </c>
+      <c r="AG30" t="s" s="2">
+        <v>81</v>
+      </c>
+      <c r="AH30" t="s" s="2">
+        <v>92</v>
+      </c>
+      <c r="AI30" t="s" s="2">
+        <v>311</v>
+      </c>
+      <c r="AJ30" t="s" s="2">
+        <v>104</v>
+      </c>
+      <c r="AK30" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="AL30" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="AM30" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="AN30" t="s" s="2">
         <v>312</v>
       </c>
-      <c r="AG30" t="s" s="2">
-        <v>81</v>
-      </c>
-      <c r="AH30" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AI30" t="s" s="2">
-        <v>80</v>
-      </c>
-      <c r="AJ30" t="s" s="2">
-        <v>316</v>
-      </c>
-      <c r="AK30" t="s" s="2">
-        <v>80</v>
-      </c>
-      <c r="AL30" t="s" s="2">
-        <v>80</v>
-      </c>
-      <c r="AM30" t="s" s="2">
-        <v>80</v>
-      </c>
-      <c r="AN30" t="s" s="2">
-        <v>317</v>
-      </c>
       <c r="AO30" t="s" s="2">
-        <v>80</v>
+        <v>313</v>
       </c>
       <c r="AP30" t="s" s="2">
         <v>80</v>
@@ -5159,10 +5230,10 @@
     </row>
     <row r="31" hidden="true">
       <c r="A31" t="s" s="2">
-        <v>318</v>
+        <v>314</v>
       </c>
       <c r="B31" t="s" s="2">
-        <v>318</v>
+        <v>314</v>
       </c>
       <c r="C31" s="2"/>
       <c r="D31" t="s" s="2">
@@ -5182,16 +5253,16 @@
         <v>80</v>
       </c>
       <c r="J31" t="s" s="2">
-        <v>80</v>
+        <v>93</v>
       </c>
       <c r="K31" t="s" s="2">
-        <v>152</v>
+        <v>315</v>
       </c>
       <c r="L31" t="s" s="2">
-        <v>153</v>
+        <v>316</v>
       </c>
       <c r="M31" t="s" s="2">
-        <v>154</v>
+        <v>317</v>
       </c>
       <c r="N31" s="2"/>
       <c r="O31" s="2"/>
@@ -5242,7 +5313,7 @@
         <v>80</v>
       </c>
       <c r="AF31" t="s" s="2">
-        <v>155</v>
+        <v>314</v>
       </c>
       <c r="AG31" t="s" s="2">
         <v>81</v>
@@ -5254,7 +5325,7 @@
         <v>80</v>
       </c>
       <c r="AJ31" t="s" s="2">
-        <v>80</v>
+        <v>104</v>
       </c>
       <c r="AK31" t="s" s="2">
         <v>80</v>
@@ -5263,13 +5334,13 @@
         <v>80</v>
       </c>
       <c r="AM31" t="s" s="2">
-        <v>80</v>
+        <v>318</v>
       </c>
       <c r="AN31" t="s" s="2">
-        <v>156</v>
+        <v>319</v>
       </c>
       <c r="AO31" t="s" s="2">
-        <v>80</v>
+        <v>320</v>
       </c>
       <c r="AP31" t="s" s="2">
         <v>80</v>
@@ -5277,21 +5348,21 @@
     </row>
     <row r="32" hidden="true">
       <c r="A32" t="s" s="2">
-        <v>319</v>
+        <v>321</v>
       </c>
       <c r="B32" t="s" s="2">
-        <v>319</v>
+        <v>321</v>
       </c>
       <c r="C32" s="2"/>
       <c r="D32" t="s" s="2">
-        <v>175</v>
+        <v>80</v>
       </c>
       <c r="E32" s="2"/>
       <c r="F32" t="s" s="2">
         <v>81</v>
       </c>
       <c r="G32" t="s" s="2">
-        <v>82</v>
+        <v>92</v>
       </c>
       <c r="H32" t="s" s="2">
         <v>80</v>
@@ -5300,20 +5371,18 @@
         <v>80</v>
       </c>
       <c r="J32" t="s" s="2">
-        <v>80</v>
+        <v>93</v>
       </c>
       <c r="K32" t="s" s="2">
-        <v>137</v>
+        <v>322</v>
       </c>
       <c r="L32" t="s" s="2">
-        <v>320</v>
+        <v>323</v>
       </c>
       <c r="M32" t="s" s="2">
-        <v>321</v>
-      </c>
-      <c r="N32" t="s" s="2">
-        <v>178</v>
-      </c>
+        <v>324</v>
+      </c>
+      <c r="N32" s="2"/>
       <c r="O32" s="2"/>
       <c r="P32" t="s" s="2">
         <v>80</v>
@@ -5362,19 +5431,19 @@
         <v>80</v>
       </c>
       <c r="AF32" t="s" s="2">
-        <v>160</v>
+        <v>321</v>
       </c>
       <c r="AG32" t="s" s="2">
         <v>81</v>
       </c>
       <c r="AH32" t="s" s="2">
-        <v>82</v>
+        <v>92</v>
       </c>
       <c r="AI32" t="s" s="2">
         <v>80</v>
       </c>
       <c r="AJ32" t="s" s="2">
-        <v>143</v>
+        <v>104</v>
       </c>
       <c r="AK32" t="s" s="2">
         <v>80</v>
@@ -5386,10 +5455,10 @@
         <v>80</v>
       </c>
       <c r="AN32" t="s" s="2">
-        <v>156</v>
+        <v>325</v>
       </c>
       <c r="AO32" t="s" s="2">
-        <v>80</v>
+        <v>326</v>
       </c>
       <c r="AP32" t="s" s="2">
         <v>80</v>
@@ -5397,46 +5466,42 @@
     </row>
     <row r="33" hidden="true">
       <c r="A33" t="s" s="2">
-        <v>322</v>
+        <v>327</v>
       </c>
       <c r="B33" t="s" s="2">
-        <v>322</v>
+        <v>327</v>
       </c>
       <c r="C33" s="2"/>
       <c r="D33" t="s" s="2">
-        <v>323</v>
+        <v>80</v>
       </c>
       <c r="E33" s="2"/>
       <c r="F33" t="s" s="2">
         <v>81</v>
       </c>
       <c r="G33" t="s" s="2">
-        <v>82</v>
+        <v>92</v>
       </c>
       <c r="H33" t="s" s="2">
         <v>80</v>
       </c>
       <c r="I33" t="s" s="2">
-        <v>93</v>
+        <v>80</v>
       </c>
       <c r="J33" t="s" s="2">
         <v>93</v>
       </c>
       <c r="K33" t="s" s="2">
-        <v>137</v>
+        <v>322</v>
       </c>
       <c r="L33" t="s" s="2">
-        <v>324</v>
+        <v>328</v>
       </c>
       <c r="M33" t="s" s="2">
-        <v>325</v>
-      </c>
-      <c r="N33" t="s" s="2">
-        <v>178</v>
-      </c>
-      <c r="O33" t="s" s="2">
-        <v>179</v>
-      </c>
+        <v>329</v>
+      </c>
+      <c r="N33" s="2"/>
+      <c r="O33" s="2"/>
       <c r="P33" t="s" s="2">
         <v>80</v>
       </c>
@@ -5484,19 +5549,19 @@
         <v>80</v>
       </c>
       <c r="AF33" t="s" s="2">
-        <v>326</v>
+        <v>327</v>
       </c>
       <c r="AG33" t="s" s="2">
         <v>81</v>
       </c>
       <c r="AH33" t="s" s="2">
-        <v>82</v>
+        <v>92</v>
       </c>
       <c r="AI33" t="s" s="2">
         <v>80</v>
       </c>
       <c r="AJ33" t="s" s="2">
-        <v>143</v>
+        <v>104</v>
       </c>
       <c r="AK33" t="s" s="2">
         <v>80</v>
@@ -5505,13 +5570,13 @@
         <v>80</v>
       </c>
       <c r="AM33" t="s" s="2">
-        <v>80</v>
+        <v>330</v>
       </c>
       <c r="AN33" t="s" s="2">
-        <v>135</v>
+        <v>331</v>
       </c>
       <c r="AO33" t="s" s="2">
-        <v>80</v>
+        <v>332</v>
       </c>
       <c r="AP33" t="s" s="2">
         <v>80</v>
@@ -5519,10 +5584,10 @@
     </row>
     <row r="34" hidden="true">
       <c r="A34" t="s" s="2">
-        <v>327</v>
+        <v>333</v>
       </c>
       <c r="B34" t="s" s="2">
-        <v>327</v>
+        <v>333</v>
       </c>
       <c r="C34" s="2"/>
       <c r="D34" t="s" s="2">
@@ -5533,7 +5598,7 @@
         <v>81</v>
       </c>
       <c r="G34" t="s" s="2">
-        <v>92</v>
+        <v>82</v>
       </c>
       <c r="H34" t="s" s="2">
         <v>80</v>
@@ -5545,13 +5610,13 @@
         <v>80</v>
       </c>
       <c r="K34" t="s" s="2">
-        <v>191</v>
+        <v>334</v>
       </c>
       <c r="L34" t="s" s="2">
-        <v>328</v>
+        <v>335</v>
       </c>
       <c r="M34" t="s" s="2">
-        <v>329</v>
+        <v>336</v>
       </c>
       <c r="N34" s="2"/>
       <c r="O34" s="2"/>
@@ -5578,13 +5643,13 @@
         <v>80</v>
       </c>
       <c r="X34" t="s" s="2">
-        <v>240</v>
+        <v>80</v>
       </c>
       <c r="Y34" t="s" s="2">
-        <v>330</v>
+        <v>80</v>
       </c>
       <c r="Z34" t="s" s="2">
-        <v>331</v>
+        <v>80</v>
       </c>
       <c r="AA34" t="s" s="2">
         <v>80</v>
@@ -5602,31 +5667,31 @@
         <v>80</v>
       </c>
       <c r="AF34" t="s" s="2">
-        <v>327</v>
+        <v>333</v>
       </c>
       <c r="AG34" t="s" s="2">
         <v>81</v>
       </c>
       <c r="AH34" t="s" s="2">
-        <v>92</v>
+        <v>82</v>
       </c>
       <c r="AI34" t="s" s="2">
-        <v>332</v>
+        <v>80</v>
       </c>
       <c r="AJ34" t="s" s="2">
-        <v>104</v>
+        <v>337</v>
       </c>
       <c r="AK34" t="s" s="2">
         <v>80</v>
       </c>
       <c r="AL34" t="s" s="2">
-        <v>333</v>
+        <v>80</v>
       </c>
       <c r="AM34" t="s" s="2">
-        <v>201</v>
+        <v>80</v>
       </c>
       <c r="AN34" t="s" s="2">
-        <v>246</v>
+        <v>338</v>
       </c>
       <c r="AO34" t="s" s="2">
         <v>80</v>
@@ -5637,10 +5702,10 @@
     </row>
     <row r="35" hidden="true">
       <c r="A35" t="s" s="2">
-        <v>334</v>
+        <v>339</v>
       </c>
       <c r="B35" t="s" s="2">
-        <v>334</v>
+        <v>339</v>
       </c>
       <c r="C35" s="2"/>
       <c r="D35" t="s" s="2">
@@ -5651,7 +5716,7 @@
         <v>81</v>
       </c>
       <c r="G35" t="s" s="2">
-        <v>82</v>
+        <v>92</v>
       </c>
       <c r="H35" t="s" s="2">
         <v>80</v>
@@ -5663,13 +5728,13 @@
         <v>80</v>
       </c>
       <c r="K35" t="s" s="2">
-        <v>335</v>
+        <v>227</v>
       </c>
       <c r="L35" t="s" s="2">
-        <v>336</v>
+        <v>228</v>
       </c>
       <c r="M35" t="s" s="2">
-        <v>337</v>
+        <v>229</v>
       </c>
       <c r="N35" s="2"/>
       <c r="O35" s="2"/>
@@ -5720,19 +5785,19 @@
         <v>80</v>
       </c>
       <c r="AF35" t="s" s="2">
-        <v>334</v>
+        <v>230</v>
       </c>
       <c r="AG35" t="s" s="2">
         <v>81</v>
       </c>
       <c r="AH35" t="s" s="2">
-        <v>82</v>
+        <v>92</v>
       </c>
       <c r="AI35" t="s" s="2">
-        <v>332</v>
+        <v>80</v>
       </c>
       <c r="AJ35" t="s" s="2">
-        <v>104</v>
+        <v>80</v>
       </c>
       <c r="AK35" t="s" s="2">
         <v>80</v>
@@ -5744,7 +5809,7 @@
         <v>80</v>
       </c>
       <c r="AN35" t="s" s="2">
-        <v>338</v>
+        <v>231</v>
       </c>
       <c r="AO35" t="s" s="2">
         <v>80</v>
@@ -5755,21 +5820,21 @@
     </row>
     <row r="36" hidden="true">
       <c r="A36" t="s" s="2">
-        <v>339</v>
+        <v>340</v>
       </c>
       <c r="B36" t="s" s="2">
-        <v>339</v>
+        <v>340</v>
       </c>
       <c r="C36" s="2"/>
       <c r="D36" t="s" s="2">
-        <v>80</v>
+        <v>137</v>
       </c>
       <c r="E36" s="2"/>
       <c r="F36" t="s" s="2">
         <v>81</v>
       </c>
       <c r="G36" t="s" s="2">
-        <v>92</v>
+        <v>82</v>
       </c>
       <c r="H36" t="s" s="2">
         <v>80</v>
@@ -5781,15 +5846,17 @@
         <v>80</v>
       </c>
       <c r="K36" t="s" s="2">
-        <v>191</v>
+        <v>138</v>
       </c>
       <c r="L36" t="s" s="2">
-        <v>340</v>
+        <v>139</v>
       </c>
       <c r="M36" t="s" s="2">
-        <v>341</v>
-      </c>
-      <c r="N36" s="2"/>
+        <v>233</v>
+      </c>
+      <c r="N36" t="s" s="2">
+        <v>141</v>
+      </c>
       <c r="O36" s="2"/>
       <c r="P36" t="s" s="2">
         <v>80</v>
@@ -5814,13 +5881,13 @@
         <v>80</v>
       </c>
       <c r="X36" t="s" s="2">
-        <v>240</v>
+        <v>80</v>
       </c>
       <c r="Y36" t="s" s="2">
-        <v>342</v>
+        <v>80</v>
       </c>
       <c r="Z36" t="s" s="2">
-        <v>343</v>
+        <v>80</v>
       </c>
       <c r="AA36" t="s" s="2">
         <v>80</v>
@@ -5838,19 +5905,19 @@
         <v>80</v>
       </c>
       <c r="AF36" t="s" s="2">
-        <v>339</v>
+        <v>237</v>
       </c>
       <c r="AG36" t="s" s="2">
         <v>81</v>
       </c>
       <c r="AH36" t="s" s="2">
-        <v>92</v>
+        <v>82</v>
       </c>
       <c r="AI36" t="s" s="2">
         <v>80</v>
       </c>
       <c r="AJ36" t="s" s="2">
-        <v>104</v>
+        <v>143</v>
       </c>
       <c r="AK36" t="s" s="2">
         <v>80</v>
@@ -5862,7 +5929,7 @@
         <v>80</v>
       </c>
       <c r="AN36" t="s" s="2">
-        <v>344</v>
+        <v>231</v>
       </c>
       <c r="AO36" t="s" s="2">
         <v>80</v>
@@ -5873,14 +5940,14 @@
     </row>
     <row r="37" hidden="true">
       <c r="A37" t="s" s="2">
-        <v>345</v>
+        <v>341</v>
       </c>
       <c r="B37" t="s" s="2">
-        <v>345</v>
+        <v>341</v>
       </c>
       <c r="C37" s="2"/>
       <c r="D37" t="s" s="2">
-        <v>80</v>
+        <v>342</v>
       </c>
       <c r="E37" s="2"/>
       <c r="F37" t="s" s="2">
@@ -5893,24 +5960,26 @@
         <v>80</v>
       </c>
       <c r="I37" t="s" s="2">
-        <v>80</v>
+        <v>93</v>
       </c>
       <c r="J37" t="s" s="2">
-        <v>80</v>
+        <v>93</v>
       </c>
       <c r="K37" t="s" s="2">
-        <v>313</v>
+        <v>138</v>
       </c>
       <c r="L37" t="s" s="2">
-        <v>346</v>
+        <v>343</v>
       </c>
       <c r="M37" t="s" s="2">
-        <v>347</v>
+        <v>344</v>
       </c>
       <c r="N37" t="s" s="2">
-        <v>348</v>
-      </c>
-      <c r="O37" s="2"/>
+        <v>141</v>
+      </c>
+      <c r="O37" t="s" s="2">
+        <v>147</v>
+      </c>
       <c r="P37" t="s" s="2">
         <v>80</v>
       </c>
@@ -5970,7 +6039,7 @@
         <v>80</v>
       </c>
       <c r="AJ37" t="s" s="2">
-        <v>349</v>
+        <v>143</v>
       </c>
       <c r="AK37" t="s" s="2">
         <v>80</v>
@@ -5982,7 +6051,7 @@
         <v>80</v>
       </c>
       <c r="AN37" t="s" s="2">
-        <v>350</v>
+        <v>135</v>
       </c>
       <c r="AO37" t="s" s="2">
         <v>80</v>
@@ -5993,10 +6062,10 @@
     </row>
     <row r="38" hidden="true">
       <c r="A38" t="s" s="2">
-        <v>351</v>
+        <v>346</v>
       </c>
       <c r="B38" t="s" s="2">
-        <v>351</v>
+        <v>346</v>
       </c>
       <c r="C38" s="2"/>
       <c r="D38" t="s" s="2">
@@ -6019,13 +6088,13 @@
         <v>80</v>
       </c>
       <c r="K38" t="s" s="2">
-        <v>152</v>
+        <v>159</v>
       </c>
       <c r="L38" t="s" s="2">
-        <v>153</v>
+        <v>347</v>
       </c>
       <c r="M38" t="s" s="2">
-        <v>154</v>
+        <v>348</v>
       </c>
       <c r="N38" s="2"/>
       <c r="O38" s="2"/>
@@ -6052,13 +6121,13 @@
         <v>80</v>
       </c>
       <c r="X38" t="s" s="2">
-        <v>80</v>
+        <v>208</v>
       </c>
       <c r="Y38" t="s" s="2">
-        <v>80</v>
+        <v>349</v>
       </c>
       <c r="Z38" t="s" s="2">
-        <v>80</v>
+        <v>350</v>
       </c>
       <c r="AA38" t="s" s="2">
         <v>80</v>
@@ -6076,7 +6145,7 @@
         <v>80</v>
       </c>
       <c r="AF38" t="s" s="2">
-        <v>155</v>
+        <v>346</v>
       </c>
       <c r="AG38" t="s" s="2">
         <v>81</v>
@@ -6085,22 +6154,22 @@
         <v>92</v>
       </c>
       <c r="AI38" t="s" s="2">
-        <v>80</v>
+        <v>351</v>
       </c>
       <c r="AJ38" t="s" s="2">
-        <v>80</v>
+        <v>104</v>
       </c>
       <c r="AK38" t="s" s="2">
         <v>80</v>
       </c>
       <c r="AL38" t="s" s="2">
-        <v>80</v>
+        <v>352</v>
       </c>
       <c r="AM38" t="s" s="2">
-        <v>80</v>
+        <v>169</v>
       </c>
       <c r="AN38" t="s" s="2">
-        <v>156</v>
+        <v>214</v>
       </c>
       <c r="AO38" t="s" s="2">
         <v>80</v>
@@ -6111,14 +6180,14 @@
     </row>
     <row r="39" hidden="true">
       <c r="A39" t="s" s="2">
-        <v>352</v>
+        <v>353</v>
       </c>
       <c r="B39" t="s" s="2">
-        <v>352</v>
+        <v>353</v>
       </c>
       <c r="C39" s="2"/>
       <c r="D39" t="s" s="2">
-        <v>175</v>
+        <v>80</v>
       </c>
       <c r="E39" s="2"/>
       <c r="F39" t="s" s="2">
@@ -6137,17 +6206,15 @@
         <v>80</v>
       </c>
       <c r="K39" t="s" s="2">
-        <v>137</v>
+        <v>354</v>
       </c>
       <c r="L39" t="s" s="2">
-        <v>320</v>
+        <v>355</v>
       </c>
       <c r="M39" t="s" s="2">
-        <v>321</v>
-      </c>
-      <c r="N39" t="s" s="2">
-        <v>178</v>
-      </c>
+        <v>356</v>
+      </c>
+      <c r="N39" s="2"/>
       <c r="O39" s="2"/>
       <c r="P39" t="s" s="2">
         <v>80</v>
@@ -6196,7 +6263,7 @@
         <v>80</v>
       </c>
       <c r="AF39" t="s" s="2">
-        <v>160</v>
+        <v>353</v>
       </c>
       <c r="AG39" t="s" s="2">
         <v>81</v>
@@ -6205,10 +6272,10 @@
         <v>82</v>
       </c>
       <c r="AI39" t="s" s="2">
-        <v>80</v>
+        <v>351</v>
       </c>
       <c r="AJ39" t="s" s="2">
-        <v>143</v>
+        <v>104</v>
       </c>
       <c r="AK39" t="s" s="2">
         <v>80</v>
@@ -6220,7 +6287,7 @@
         <v>80</v>
       </c>
       <c r="AN39" t="s" s="2">
-        <v>156</v>
+        <v>357</v>
       </c>
       <c r="AO39" t="s" s="2">
         <v>80</v>
@@ -6231,46 +6298,42 @@
     </row>
     <row r="40" hidden="true">
       <c r="A40" t="s" s="2">
-        <v>353</v>
+        <v>358</v>
       </c>
       <c r="B40" t="s" s="2">
-        <v>353</v>
+        <v>358</v>
       </c>
       <c r="C40" s="2"/>
       <c r="D40" t="s" s="2">
-        <v>323</v>
+        <v>80</v>
       </c>
       <c r="E40" s="2"/>
       <c r="F40" t="s" s="2">
         <v>81</v>
       </c>
       <c r="G40" t="s" s="2">
-        <v>82</v>
+        <v>92</v>
       </c>
       <c r="H40" t="s" s="2">
         <v>80</v>
       </c>
       <c r="I40" t="s" s="2">
-        <v>93</v>
+        <v>80</v>
       </c>
       <c r="J40" t="s" s="2">
-        <v>93</v>
+        <v>80</v>
       </c>
       <c r="K40" t="s" s="2">
-        <v>137</v>
+        <v>159</v>
       </c>
       <c r="L40" t="s" s="2">
-        <v>324</v>
+        <v>359</v>
       </c>
       <c r="M40" t="s" s="2">
-        <v>325</v>
-      </c>
-      <c r="N40" t="s" s="2">
-        <v>178</v>
-      </c>
-      <c r="O40" t="s" s="2">
-        <v>179</v>
-      </c>
+        <v>360</v>
+      </c>
+      <c r="N40" s="2"/>
+      <c r="O40" s="2"/>
       <c r="P40" t="s" s="2">
         <v>80</v>
       </c>
@@ -6294,13 +6357,13 @@
         <v>80</v>
       </c>
       <c r="X40" t="s" s="2">
-        <v>80</v>
+        <v>208</v>
       </c>
       <c r="Y40" t="s" s="2">
-        <v>80</v>
+        <v>361</v>
       </c>
       <c r="Z40" t="s" s="2">
-        <v>80</v>
+        <v>362</v>
       </c>
       <c r="AA40" t="s" s="2">
         <v>80</v>
@@ -6318,19 +6381,19 @@
         <v>80</v>
       </c>
       <c r="AF40" t="s" s="2">
-        <v>326</v>
+        <v>358</v>
       </c>
       <c r="AG40" t="s" s="2">
         <v>81</v>
       </c>
       <c r="AH40" t="s" s="2">
-        <v>82</v>
+        <v>92</v>
       </c>
       <c r="AI40" t="s" s="2">
         <v>80</v>
       </c>
       <c r="AJ40" t="s" s="2">
-        <v>143</v>
+        <v>104</v>
       </c>
       <c r="AK40" t="s" s="2">
         <v>80</v>
@@ -6342,7 +6405,7 @@
         <v>80</v>
       </c>
       <c r="AN40" t="s" s="2">
-        <v>135</v>
+        <v>363</v>
       </c>
       <c r="AO40" t="s" s="2">
         <v>80</v>
@@ -6353,10 +6416,10 @@
     </row>
     <row r="41" hidden="true">
       <c r="A41" t="s" s="2">
-        <v>354</v>
+        <v>364</v>
       </c>
       <c r="B41" t="s" s="2">
-        <v>354</v>
+        <v>364</v>
       </c>
       <c r="C41" s="2"/>
       <c r="D41" t="s" s="2">
@@ -6376,18 +6439,20 @@
         <v>80</v>
       </c>
       <c r="J41" t="s" s="2">
-        <v>93</v>
+        <v>80</v>
       </c>
       <c r="K41" t="s" s="2">
-        <v>191</v>
+        <v>334</v>
       </c>
       <c r="L41" t="s" s="2">
-        <v>355</v>
+        <v>365</v>
       </c>
       <c r="M41" t="s" s="2">
-        <v>356</v>
-      </c>
-      <c r="N41" s="2"/>
+        <v>366</v>
+      </c>
+      <c r="N41" t="s" s="2">
+        <v>367</v>
+      </c>
       <c r="O41" s="2"/>
       <c r="P41" t="s" s="2">
         <v>80</v>
@@ -6412,13 +6477,13 @@
         <v>80</v>
       </c>
       <c r="X41" t="s" s="2">
-        <v>240</v>
+        <v>80</v>
       </c>
       <c r="Y41" t="s" s="2">
-        <v>357</v>
+        <v>80</v>
       </c>
       <c r="Z41" t="s" s="2">
-        <v>358</v>
+        <v>80</v>
       </c>
       <c r="AA41" t="s" s="2">
         <v>80</v>
@@ -6436,7 +6501,7 @@
         <v>80</v>
       </c>
       <c r="AF41" t="s" s="2">
-        <v>354</v>
+        <v>364</v>
       </c>
       <c r="AG41" t="s" s="2">
         <v>81</v>
@@ -6445,25 +6510,25 @@
         <v>82</v>
       </c>
       <c r="AI41" t="s" s="2">
-        <v>359</v>
+        <v>80</v>
       </c>
       <c r="AJ41" t="s" s="2">
-        <v>104</v>
+        <v>368</v>
       </c>
       <c r="AK41" t="s" s="2">
-        <v>360</v>
+        <v>80</v>
       </c>
       <c r="AL41" t="s" s="2">
-        <v>221</v>
+        <v>80</v>
       </c>
       <c r="AM41" t="s" s="2">
         <v>80</v>
       </c>
       <c r="AN41" t="s" s="2">
-        <v>361</v>
+        <v>369</v>
       </c>
       <c r="AO41" t="s" s="2">
-        <v>362</v>
+        <v>80</v>
       </c>
       <c r="AP41" t="s" s="2">
         <v>80</v>
@@ -6471,10 +6536,10 @@
     </row>
     <row r="42" hidden="true">
       <c r="A42" t="s" s="2">
-        <v>363</v>
+        <v>370</v>
       </c>
       <c r="B42" t="s" s="2">
-        <v>363</v>
+        <v>370</v>
       </c>
       <c r="C42" s="2"/>
       <c r="D42" t="s" s="2">
@@ -6485,7 +6550,7 @@
         <v>81</v>
       </c>
       <c r="G42" t="s" s="2">
-        <v>82</v>
+        <v>92</v>
       </c>
       <c r="H42" t="s" s="2">
         <v>80</v>
@@ -6494,16 +6559,16 @@
         <v>80</v>
       </c>
       <c r="J42" t="s" s="2">
-        <v>93</v>
+        <v>80</v>
       </c>
       <c r="K42" t="s" s="2">
-        <v>364</v>
+        <v>227</v>
       </c>
       <c r="L42" t="s" s="2">
-        <v>365</v>
+        <v>228</v>
       </c>
       <c r="M42" t="s" s="2">
-        <v>366</v>
+        <v>229</v>
       </c>
       <c r="N42" s="2"/>
       <c r="O42" s="2"/>
@@ -6554,19 +6619,19 @@
         <v>80</v>
       </c>
       <c r="AF42" t="s" s="2">
-        <v>363</v>
+        <v>230</v>
       </c>
       <c r="AG42" t="s" s="2">
         <v>81</v>
       </c>
       <c r="AH42" t="s" s="2">
-        <v>82</v>
+        <v>92</v>
       </c>
       <c r="AI42" t="s" s="2">
-        <v>359</v>
+        <v>80</v>
       </c>
       <c r="AJ42" t="s" s="2">
-        <v>104</v>
+        <v>80</v>
       </c>
       <c r="AK42" t="s" s="2">
         <v>80</v>
@@ -6578,10 +6643,10 @@
         <v>80</v>
       </c>
       <c r="AN42" t="s" s="2">
-        <v>338</v>
+        <v>231</v>
       </c>
       <c r="AO42" t="s" s="2">
-        <v>362</v>
+        <v>80</v>
       </c>
       <c r="AP42" t="s" s="2">
         <v>80</v>
@@ -6589,14 +6654,14 @@
     </row>
     <row r="43" hidden="true">
       <c r="A43" t="s" s="2">
-        <v>367</v>
+        <v>371</v>
       </c>
       <c r="B43" t="s" s="2">
-        <v>367</v>
+        <v>371</v>
       </c>
       <c r="C43" s="2"/>
       <c r="D43" t="s" s="2">
-        <v>80</v>
+        <v>137</v>
       </c>
       <c r="E43" s="2"/>
       <c r="F43" t="s" s="2">
@@ -6615,15 +6680,17 @@
         <v>80</v>
       </c>
       <c r="K43" t="s" s="2">
-        <v>368</v>
+        <v>138</v>
       </c>
       <c r="L43" t="s" s="2">
-        <v>369</v>
+        <v>139</v>
       </c>
       <c r="M43" t="s" s="2">
-        <v>370</v>
-      </c>
-      <c r="N43" s="2"/>
+        <v>233</v>
+      </c>
+      <c r="N43" t="s" s="2">
+        <v>141</v>
+      </c>
       <c r="O43" s="2"/>
       <c r="P43" t="s" s="2">
         <v>80</v>
@@ -6672,7 +6739,7 @@
         <v>80</v>
       </c>
       <c r="AF43" t="s" s="2">
-        <v>367</v>
+        <v>237</v>
       </c>
       <c r="AG43" t="s" s="2">
         <v>81</v>
@@ -6684,29 +6751,505 @@
         <v>80</v>
       </c>
       <c r="AJ43" t="s" s="2">
+        <v>143</v>
+      </c>
+      <c r="AK43" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="AL43" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="AM43" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="AN43" t="s" s="2">
+        <v>231</v>
+      </c>
+      <c r="AO43" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="AP43" t="s" s="2">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="44" hidden="true">
+      <c r="A44" t="s" s="2">
+        <v>372</v>
+      </c>
+      <c r="B44" t="s" s="2">
+        <v>372</v>
+      </c>
+      <c r="C44" s="2"/>
+      <c r="D44" t="s" s="2">
+        <v>342</v>
+      </c>
+      <c r="E44" s="2"/>
+      <c r="F44" t="s" s="2">
+        <v>81</v>
+      </c>
+      <c r="G44" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="H44" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="I44" t="s" s="2">
+        <v>93</v>
+      </c>
+      <c r="J44" t="s" s="2">
+        <v>93</v>
+      </c>
+      <c r="K44" t="s" s="2">
+        <v>138</v>
+      </c>
+      <c r="L44" t="s" s="2">
+        <v>343</v>
+      </c>
+      <c r="M44" t="s" s="2">
+        <v>344</v>
+      </c>
+      <c r="N44" t="s" s="2">
+        <v>141</v>
+      </c>
+      <c r="O44" t="s" s="2">
+        <v>147</v>
+      </c>
+      <c r="P44" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="Q44" s="2"/>
+      <c r="R44" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="S44" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="T44" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="U44" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="V44" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="W44" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="X44" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="Y44" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="Z44" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="AA44" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="AB44" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="AC44" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="AD44" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="AE44" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="AF44" t="s" s="2">
+        <v>345</v>
+      </c>
+      <c r="AG44" t="s" s="2">
+        <v>81</v>
+      </c>
+      <c r="AH44" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="AI44" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="AJ44" t="s" s="2">
+        <v>143</v>
+      </c>
+      <c r="AK44" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="AL44" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="AM44" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="AN44" t="s" s="2">
+        <v>135</v>
+      </c>
+      <c r="AO44" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="AP44" t="s" s="2">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="45" hidden="true">
+      <c r="A45" t="s" s="2">
+        <v>373</v>
+      </c>
+      <c r="B45" t="s" s="2">
+        <v>373</v>
+      </c>
+      <c r="C45" s="2"/>
+      <c r="D45" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="E45" s="2"/>
+      <c r="F45" t="s" s="2">
+        <v>81</v>
+      </c>
+      <c r="G45" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="H45" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="I45" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="J45" t="s" s="2">
+        <v>93</v>
+      </c>
+      <c r="K45" t="s" s="2">
+        <v>159</v>
+      </c>
+      <c r="L45" t="s" s="2">
+        <v>374</v>
+      </c>
+      <c r="M45" t="s" s="2">
+        <v>375</v>
+      </c>
+      <c r="N45" s="2"/>
+      <c r="O45" s="2"/>
+      <c r="P45" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="Q45" s="2"/>
+      <c r="R45" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="S45" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="T45" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="U45" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="V45" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="W45" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="X45" t="s" s="2">
+        <v>208</v>
+      </c>
+      <c r="Y45" t="s" s="2">
+        <v>376</v>
+      </c>
+      <c r="Z45" t="s" s="2">
+        <v>377</v>
+      </c>
+      <c r="AA45" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="AB45" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="AC45" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="AD45" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="AE45" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="AF45" t="s" s="2">
+        <v>373</v>
+      </c>
+      <c r="AG45" t="s" s="2">
+        <v>81</v>
+      </c>
+      <c r="AH45" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="AI45" t="s" s="2">
+        <v>378</v>
+      </c>
+      <c r="AJ45" t="s" s="2">
         <v>104</v>
       </c>
-      <c r="AK43" t="s" s="2">
-        <v>371</v>
-      </c>
-      <c r="AL43" t="s" s="2">
-        <v>80</v>
-      </c>
-      <c r="AM43" t="s" s="2">
-        <v>372</v>
-      </c>
-      <c r="AN43" t="s" s="2">
-        <v>373</v>
-      </c>
-      <c r="AO43" t="s" s="2">
-        <v>80</v>
-      </c>
-      <c r="AP43" t="s" s="2">
+      <c r="AK45" t="s" s="2">
+        <v>379</v>
+      </c>
+      <c r="AL45" t="s" s="2">
+        <v>189</v>
+      </c>
+      <c r="AM45" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="AN45" t="s" s="2">
+        <v>380</v>
+      </c>
+      <c r="AO45" t="s" s="2">
+        <v>381</v>
+      </c>
+      <c r="AP45" t="s" s="2">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="46" hidden="true">
+      <c r="A46" t="s" s="2">
+        <v>382</v>
+      </c>
+      <c r="B46" t="s" s="2">
+        <v>382</v>
+      </c>
+      <c r="C46" s="2"/>
+      <c r="D46" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="E46" s="2"/>
+      <c r="F46" t="s" s="2">
+        <v>81</v>
+      </c>
+      <c r="G46" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="H46" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="I46" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="J46" t="s" s="2">
+        <v>93</v>
+      </c>
+      <c r="K46" t="s" s="2">
+        <v>383</v>
+      </c>
+      <c r="L46" t="s" s="2">
+        <v>384</v>
+      </c>
+      <c r="M46" t="s" s="2">
+        <v>385</v>
+      </c>
+      <c r="N46" s="2"/>
+      <c r="O46" s="2"/>
+      <c r="P46" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="Q46" s="2"/>
+      <c r="R46" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="S46" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="T46" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="U46" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="V46" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="W46" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="X46" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="Y46" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="Z46" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="AA46" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="AB46" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="AC46" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="AD46" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="AE46" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="AF46" t="s" s="2">
+        <v>382</v>
+      </c>
+      <c r="AG46" t="s" s="2">
+        <v>81</v>
+      </c>
+      <c r="AH46" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="AI46" t="s" s="2">
+        <v>378</v>
+      </c>
+      <c r="AJ46" t="s" s="2">
+        <v>104</v>
+      </c>
+      <c r="AK46" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="AL46" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="AM46" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="AN46" t="s" s="2">
+        <v>357</v>
+      </c>
+      <c r="AO46" t="s" s="2">
+        <v>381</v>
+      </c>
+      <c r="AP46" t="s" s="2">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="47" hidden="true">
+      <c r="A47" t="s" s="2">
+        <v>386</v>
+      </c>
+      <c r="B47" t="s" s="2">
+        <v>386</v>
+      </c>
+      <c r="C47" s="2"/>
+      <c r="D47" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="E47" s="2"/>
+      <c r="F47" t="s" s="2">
+        <v>81</v>
+      </c>
+      <c r="G47" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="H47" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="I47" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="J47" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="K47" t="s" s="2">
+        <v>387</v>
+      </c>
+      <c r="L47" t="s" s="2">
+        <v>388</v>
+      </c>
+      <c r="M47" t="s" s="2">
+        <v>389</v>
+      </c>
+      <c r="N47" s="2"/>
+      <c r="O47" s="2"/>
+      <c r="P47" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="Q47" s="2"/>
+      <c r="R47" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="S47" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="T47" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="U47" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="V47" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="W47" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="X47" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="Y47" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="Z47" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="AA47" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="AB47" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="AC47" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="AD47" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="AE47" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="AF47" t="s" s="2">
+        <v>386</v>
+      </c>
+      <c r="AG47" t="s" s="2">
+        <v>81</v>
+      </c>
+      <c r="AH47" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="AI47" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="AJ47" t="s" s="2">
+        <v>104</v>
+      </c>
+      <c r="AK47" t="s" s="2">
+        <v>390</v>
+      </c>
+      <c r="AL47" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="AM47" t="s" s="2">
+        <v>391</v>
+      </c>
+      <c r="AN47" t="s" s="2">
+        <v>392</v>
+      </c>
+      <c r="AO47" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="AP47" t="s" s="2">
         <v>80</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:AP43">
+  <autoFilter ref="A1:AP47">
     <filterColumn colId="7">
       <customFilters>
         <customFilter operator="notEqual" val=" "/>
@@ -6716,7 +7259,7 @@
       <filters blank="true"/>
     </filterColumn>
   </autoFilter>
-  <conditionalFormatting sqref="A2:AI42">
+  <conditionalFormatting sqref="A2:AI46">
     <cfRule type="expression" dxfId="0" priority="1">
       <formula>$G2&lt;&gt;"Y"</formula>
     </cfRule>

</xml_diff>